<commit_message>
ADD: new prices from 06.04.2026
</commit_message>
<xml_diff>
--- a/A_FINAL_RESULT/eko_transactions.xlsx
+++ b/A_FINAL_RESULT/eko_transactions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\A_FINAL_RESULT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B9B4239-90E6-4CE9-AFF1-74514A300C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CAA947F-4CAE-4717-935B-F72CFC6E46AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="35" activeTab="37" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="АГРАРЕН УНИВЕРСИТЕТ - ПЛОВДИВ" sheetId="1" r:id="rId1"/>
@@ -32,9 +32,9 @@
     <sheet name="ДОК ТРАНС ЕООД" sheetId="17" r:id="rId17"/>
     <sheet name="ЕВРО ТРАНС ПРЕМИУМ ЕООД" sheetId="18" r:id="rId18"/>
     <sheet name="ЕВРОУЕЙ СЪРВИЗ ООД" sheetId="19" r:id="rId19"/>
-    <sheet name="ЖЕЛЯЗКОВ ИНЖЕНЕРИНГ - ПРОИЗВОДС" sheetId="20" r:id="rId20"/>
-    <sheet name="ЖИВКО НЕДЕЛЧЕВ ДИМИТРОВ" sheetId="21" r:id="rId21"/>
-    <sheet name="ЗЕМЕДЕЛСКА ТЕХНИКА ООД" sheetId="22" r:id="rId22"/>
+    <sheet name="ЖИВКО НЕДЕЛЧЕВ ДИМИТРОВ" sheetId="21" r:id="rId20"/>
+    <sheet name="ЗЕМЕДЕЛСКА ТЕХНИКА ООД" sheetId="22" r:id="rId21"/>
+    <sheet name="ЖЕЛЯЗКОВ ИНЖЕНЕРИНГ - ПРОИЗВОДС" sheetId="20" r:id="rId22"/>
     <sheet name="ЗП ВЕСЕЛИН СТЕФАНОВ ЖЕЛЯЗКОВ" sheetId="23" r:id="rId23"/>
     <sheet name="ИВО ИВАНОВ ЧЗС" sheetId="24" r:id="rId24"/>
     <sheet name="ИВОН СТРОЙ 2015 ЕООД" sheetId="25" r:id="rId25"/>
@@ -58,7 +58,7 @@
     <sheet name="ХРАНИНВЕСТ ЕООД % ТЪРГОВЦИ" sheetId="43" r:id="rId43"/>
     <sheet name="Unknown" sheetId="44" r:id="rId44"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
@@ -5025,10 +5025,15 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -5653,8 +5658,18 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -13323,8 +13338,8 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
-  <dimension ref="A1:M19"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -13370,239 +13385,209 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="B2" t="s">
-        <v>432</v>
+        <v>380</v>
       </c>
       <c r="C2" t="s">
-        <v>602</v>
+        <v>625</v>
       </c>
       <c r="D2" t="s">
-        <v>603</v>
+        <v>626</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>240</v>
       </c>
       <c r="F2">
-        <v>42.976999999999897</v>
+        <v>37.261000000000003</v>
       </c>
       <c r="G2" t="s">
         <v>18</v>
       </c>
-      <c r="H2">
-        <v>1.21</v>
-      </c>
-      <c r="I2">
-        <v>52</v>
-      </c>
       <c r="J2">
-        <v>1.31</v>
+        <v>1.53</v>
       </c>
       <c r="K2">
-        <v>56.3</v>
+        <v>57.01</v>
       </c>
       <c r="L2" t="s">
-        <v>604</v>
+        <v>627</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>15671</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>432</v>
       </c>
       <c r="C3" t="s">
-        <v>605</v>
+        <v>628</v>
       </c>
       <c r="D3" t="s">
-        <v>606</v>
+        <v>629</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>240</v>
       </c>
       <c r="F3">
-        <v>40.137</v>
+        <v>26.707999999999899</v>
       </c>
       <c r="G3" t="s">
         <v>18</v>
       </c>
-      <c r="H3">
-        <v>1.21</v>
-      </c>
-      <c r="I3">
-        <v>48.57</v>
-      </c>
       <c r="J3">
-        <v>1.31</v>
+        <v>1.54</v>
       </c>
       <c r="K3">
-        <v>52.58</v>
+        <v>41.13</v>
       </c>
       <c r="L3" t="s">
-        <v>607</v>
+        <v>630</v>
       </c>
       <c r="M3">
-        <v>316540</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>202</v>
       </c>
       <c r="C4" t="s">
-        <v>608</v>
+        <v>625</v>
       </c>
       <c r="D4" t="s">
-        <v>609</v>
+        <v>626</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>240</v>
       </c>
       <c r="F4">
-        <v>49.811999999999898</v>
+        <v>24.859000000000002</v>
       </c>
       <c r="G4" t="s">
         <v>18</v>
       </c>
-      <c r="H4">
-        <v>1.23</v>
-      </c>
-      <c r="I4">
-        <v>61.27</v>
-      </c>
       <c r="J4">
-        <v>1.33</v>
+        <v>1.56</v>
       </c>
       <c r="K4">
-        <v>66.25</v>
+        <v>38.78</v>
       </c>
       <c r="L4" t="s">
-        <v>610</v>
+        <v>631</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>15913</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B5" t="s">
-        <v>380</v>
+        <v>432</v>
       </c>
       <c r="C5" t="s">
-        <v>605</v>
+        <v>632</v>
       </c>
       <c r="D5" t="s">
-        <v>606</v>
+        <v>633</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="F5">
-        <v>54.6099999999999</v>
+        <v>41.091000000000001</v>
       </c>
       <c r="G5" t="s">
         <v>18</v>
       </c>
-      <c r="H5">
-        <v>1.25</v>
-      </c>
-      <c r="I5">
-        <v>68.260000000000005</v>
-      </c>
       <c r="J5">
-        <v>1.41</v>
+        <v>1.32</v>
       </c>
       <c r="K5">
-        <v>77</v>
+        <v>54.24</v>
       </c>
       <c r="L5" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="M5">
-        <v>316950</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>177</v>
       </c>
       <c r="B6" t="s">
-        <v>93</v>
+        <v>436</v>
       </c>
       <c r="C6" t="s">
-        <v>608</v>
+        <v>625</v>
       </c>
       <c r="D6" t="s">
-        <v>609</v>
+        <v>626</v>
       </c>
       <c r="E6" t="s">
-        <v>179</v>
+        <v>45</v>
       </c>
       <c r="F6">
-        <v>48.088999999999899</v>
+        <v>37.563000000000002</v>
       </c>
       <c r="G6" t="s">
         <v>18</v>
       </c>
       <c r="J6">
-        <v>1.68</v>
+        <v>1.35</v>
       </c>
       <c r="K6">
-        <v>80.790000000000006</v>
+        <v>50.71</v>
       </c>
       <c r="L6" t="s">
-        <v>128</v>
+        <v>448</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>16287</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>380</v>
       </c>
       <c r="C7" t="s">
-        <v>612</v>
+        <v>628</v>
       </c>
       <c r="D7" t="s">
-        <v>613</v>
+        <v>629</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>240</v>
       </c>
       <c r="F7">
-        <v>33.817999999999898</v>
+        <v>26.739000000000001</v>
       </c>
       <c r="G7" t="s">
         <v>18</v>
       </c>
-      <c r="H7">
-        <v>1.25</v>
-      </c>
-      <c r="I7">
-        <v>42.27</v>
-      </c>
       <c r="J7">
-        <v>1.43</v>
+        <v>1.61</v>
       </c>
       <c r="K7">
-        <v>48.36</v>
+        <v>43.05</v>
       </c>
       <c r="L7" t="s">
-        <v>614</v>
+        <v>634</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -13610,163 +13595,139 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>380</v>
+        <v>252</v>
       </c>
       <c r="C8" t="s">
-        <v>605</v>
+        <v>625</v>
       </c>
       <c r="D8" t="s">
-        <v>606</v>
+        <v>626</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>240</v>
       </c>
       <c r="F8">
-        <v>20.4149999999999</v>
+        <v>28.117999999999899</v>
       </c>
       <c r="G8" t="s">
         <v>18</v>
       </c>
-      <c r="H8">
-        <v>1.42</v>
-      </c>
-      <c r="I8">
-        <v>28.99</v>
-      </c>
       <c r="J8">
-        <v>1.47</v>
+        <v>1.69</v>
       </c>
       <c r="K8">
-        <v>30.01</v>
+        <v>47.52</v>
       </c>
       <c r="L8" t="s">
-        <v>615</v>
+        <v>108</v>
       </c>
       <c r="M8">
-        <v>317270</v>
+        <v>16883</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>274</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
         <v>93</v>
       </c>
       <c r="C9" t="s">
-        <v>602</v>
+        <v>632</v>
       </c>
       <c r="D9" t="s">
-        <v>603</v>
+        <v>633</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="F9">
-        <v>36.362000000000002</v>
+        <v>43.542000000000002</v>
       </c>
       <c r="G9" t="s">
         <v>18</v>
       </c>
-      <c r="H9">
-        <v>1.46</v>
-      </c>
-      <c r="I9">
-        <v>53.09</v>
-      </c>
       <c r="J9">
-        <v>1.52</v>
+        <v>1.42</v>
       </c>
       <c r="K9">
-        <v>55.27</v>
+        <v>61.83</v>
       </c>
       <c r="L9" t="s">
-        <v>616</v>
+        <v>267</v>
       </c>
       <c r="M9">
-        <v>430120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>274</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>380</v>
+        <v>208</v>
       </c>
       <c r="C10" t="s">
-        <v>605</v>
+        <v>625</v>
       </c>
       <c r="D10" t="s">
-        <v>606</v>
+        <v>626</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>240</v>
       </c>
       <c r="F10">
-        <v>30.867999999999899</v>
+        <v>31.337</v>
       </c>
       <c r="G10" t="s">
         <v>18</v>
       </c>
-      <c r="H10">
-        <v>1.46</v>
-      </c>
-      <c r="I10">
-        <v>45.07</v>
-      </c>
       <c r="J10">
-        <v>1.51</v>
+        <v>1.69</v>
       </c>
       <c r="K10">
-        <v>46.61</v>
+        <v>52.96</v>
       </c>
       <c r="L10" t="s">
-        <v>617</v>
+        <v>635</v>
       </c>
       <c r="M10">
-        <v>317370</v>
+        <v>16562</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>84</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
+        <v>432</v>
       </c>
       <c r="C11" t="s">
-        <v>612</v>
+        <v>628</v>
       </c>
       <c r="D11" t="s">
-        <v>613</v>
+        <v>629</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>240</v>
       </c>
       <c r="F11">
-        <v>24.591999999999899</v>
+        <v>28.210999999999899</v>
       </c>
       <c r="G11" t="s">
         <v>18</v>
       </c>
-      <c r="H11">
-        <v>1.46</v>
-      </c>
-      <c r="I11">
-        <v>35.9</v>
-      </c>
       <c r="J11">
-        <v>1.52</v>
+        <v>1.71</v>
       </c>
       <c r="K11">
-        <v>37.380000000000003</v>
+        <v>48.24</v>
       </c>
       <c r="L11" t="s">
-        <v>618</v>
+        <v>547</v>
       </c>
       <c r="M11">
         <v>0</v>
@@ -13774,330 +13735,37 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>315</v>
       </c>
       <c r="B12" t="s">
-        <v>380</v>
+        <v>410</v>
       </c>
       <c r="C12" t="s">
-        <v>605</v>
+        <v>625</v>
       </c>
       <c r="D12" t="s">
-        <v>606</v>
+        <v>626</v>
       </c>
       <c r="E12" t="s">
-        <v>17</v>
+        <v>240</v>
       </c>
       <c r="F12">
-        <v>22.882000000000001</v>
+        <v>26.491</v>
       </c>
       <c r="G12" t="s">
         <v>18</v>
       </c>
-      <c r="H12">
-        <v>1.48</v>
-      </c>
-      <c r="I12">
-        <v>33.869999999999997</v>
-      </c>
       <c r="J12">
-        <v>1.53</v>
+        <v>1.73</v>
       </c>
       <c r="K12">
-        <v>35.01</v>
+        <v>45.83</v>
       </c>
       <c r="L12" t="s">
-        <v>619</v>
+        <v>636</v>
       </c>
       <c r="M12">
-        <v>317685</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>299</v>
-      </c>
-      <c r="B13" t="s">
-        <v>93</v>
-      </c>
-      <c r="C13" t="s">
-        <v>605</v>
-      </c>
-      <c r="D13" t="s">
-        <v>606</v>
-      </c>
-      <c r="E13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F13">
-        <v>44.963000000000001</v>
-      </c>
-      <c r="G13" t="s">
-        <v>18</v>
-      </c>
-      <c r="H13">
-        <v>1.54</v>
-      </c>
-      <c r="I13">
-        <v>69.239999999999995</v>
-      </c>
-      <c r="J13">
-        <v>1.6</v>
-      </c>
-      <c r="K13">
-        <v>71.94</v>
-      </c>
-      <c r="L13" t="s">
-        <v>505</v>
-      </c>
-      <c r="M13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>299</v>
-      </c>
-      <c r="B14" t="s">
-        <v>224</v>
-      </c>
-      <c r="C14" t="s">
-        <v>605</v>
-      </c>
-      <c r="D14" t="s">
-        <v>606</v>
-      </c>
-      <c r="E14" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14">
-        <v>30.207999999999899</v>
-      </c>
-      <c r="G14" t="s">
-        <v>18</v>
-      </c>
-      <c r="H14">
-        <v>1.54</v>
-      </c>
-      <c r="I14">
-        <v>46.52</v>
-      </c>
-      <c r="J14">
-        <v>1.59</v>
-      </c>
-      <c r="K14">
-        <v>48.03</v>
-      </c>
-      <c r="L14" t="s">
-        <v>620</v>
-      </c>
-      <c r="M14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>69</v>
-      </c>
-      <c r="B15" t="s">
-        <v>93</v>
-      </c>
-      <c r="C15" t="s">
-        <v>608</v>
-      </c>
-      <c r="D15" t="s">
-        <v>609</v>
-      </c>
-      <c r="E15" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15">
-        <v>48.701999999999899</v>
-      </c>
-      <c r="G15" t="s">
-        <v>18</v>
-      </c>
-      <c r="H15">
-        <v>1.6</v>
-      </c>
-      <c r="I15">
-        <v>77.92</v>
-      </c>
-      <c r="J15">
-        <v>1.61</v>
-      </c>
-      <c r="K15">
-        <v>78.41</v>
-      </c>
-      <c r="L15" t="s">
-        <v>130</v>
-      </c>
-      <c r="M15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>69</v>
-      </c>
-      <c r="B16" t="s">
-        <v>93</v>
-      </c>
-      <c r="C16" t="s">
-        <v>612</v>
-      </c>
-      <c r="D16" t="s">
-        <v>613</v>
-      </c>
-      <c r="E16" t="s">
-        <v>17</v>
-      </c>
-      <c r="F16">
-        <v>32.783000000000001</v>
-      </c>
-      <c r="G16" t="s">
-        <v>18</v>
-      </c>
-      <c r="H16">
-        <v>1.6</v>
-      </c>
-      <c r="I16">
-        <v>52.45</v>
-      </c>
-      <c r="J16">
-        <v>1.61</v>
-      </c>
-      <c r="K16">
-        <v>52.78</v>
-      </c>
-      <c r="L16" t="s">
-        <v>621</v>
-      </c>
-      <c r="M16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" t="s">
-        <v>75</v>
-      </c>
-      <c r="C17" t="s">
-        <v>602</v>
-      </c>
-      <c r="D17" t="s">
-        <v>603</v>
-      </c>
-      <c r="E17" t="s">
-        <v>17</v>
-      </c>
-      <c r="F17">
-        <v>40.512</v>
-      </c>
-      <c r="G17" t="s">
-        <v>18</v>
-      </c>
-      <c r="H17">
-        <v>1.6</v>
-      </c>
-      <c r="I17">
-        <v>64.819999999999993</v>
-      </c>
-      <c r="J17">
-        <v>1.62</v>
-      </c>
-      <c r="K17">
-        <v>65.63</v>
-      </c>
-      <c r="L17" t="s">
-        <v>622</v>
-      </c>
-      <c r="M17">
-        <v>430652</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>135</v>
-      </c>
-      <c r="B18" t="s">
-        <v>224</v>
-      </c>
-      <c r="C18" t="s">
-        <v>605</v>
-      </c>
-      <c r="D18" t="s">
-        <v>606</v>
-      </c>
-      <c r="E18" t="s">
-        <v>17</v>
-      </c>
-      <c r="F18">
-        <v>28.27</v>
-      </c>
-      <c r="G18" t="s">
-        <v>18</v>
-      </c>
-      <c r="H18">
-        <v>1.61</v>
-      </c>
-      <c r="I18">
-        <v>45.51</v>
-      </c>
-      <c r="J18">
-        <v>1.63</v>
-      </c>
-      <c r="K18">
-        <v>46.08</v>
-      </c>
-      <c r="L18" t="s">
-        <v>623</v>
-      </c>
-      <c r="M18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>72</v>
-      </c>
-      <c r="B19" t="s">
-        <v>380</v>
-      </c>
-      <c r="C19" t="s">
-        <v>605</v>
-      </c>
-      <c r="D19" t="s">
-        <v>606</v>
-      </c>
-      <c r="E19" t="s">
-        <v>17</v>
-      </c>
-      <c r="F19">
-        <v>50.142000000000003</v>
-      </c>
-      <c r="G19" t="s">
-        <v>18</v>
-      </c>
-      <c r="H19">
-        <v>1.64</v>
-      </c>
-      <c r="I19">
-        <v>82.23</v>
-      </c>
-      <c r="J19">
-        <v>1.69</v>
-      </c>
-      <c r="K19">
-        <v>84.74</v>
-      </c>
-      <c r="L19" t="s">
-        <v>624</v>
-      </c>
-      <c r="M19">
-        <v>318930</v>
+        <v>17100</v>
       </c>
     </row>
   </sheetData>
@@ -14106,9 +13774,17 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
-  <dimension ref="A1:M12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -14156,66 +13832,78 @@
         <v>104</v>
       </c>
       <c r="B2" t="s">
-        <v>380</v>
+        <v>70</v>
       </c>
       <c r="C2" t="s">
-        <v>625</v>
+        <v>637</v>
       </c>
       <c r="D2" t="s">
-        <v>626</v>
+        <v>638</v>
       </c>
       <c r="E2" t="s">
-        <v>240</v>
+        <v>17</v>
       </c>
       <c r="F2">
-        <v>37.261000000000003</v>
+        <v>62.2349999999999</v>
       </c>
       <c r="G2" t="s">
         <v>18</v>
       </c>
+      <c r="H2">
+        <v>1.21</v>
+      </c>
+      <c r="I2">
+        <v>75.3</v>
+      </c>
       <c r="J2">
-        <v>1.53</v>
+        <v>1.32</v>
       </c>
       <c r="K2">
-        <v>57.01</v>
+        <v>82.15</v>
       </c>
       <c r="L2" t="s">
-        <v>627</v>
+        <v>639</v>
       </c>
       <c r="M2">
-        <v>15671</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>107</v>
       </c>
       <c r="B3" t="s">
-        <v>432</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
-        <v>628</v>
+        <v>640</v>
       </c>
       <c r="D3" t="s">
-        <v>629</v>
+        <v>641</v>
       </c>
       <c r="E3" t="s">
-        <v>240</v>
+        <v>45</v>
       </c>
       <c r="F3">
-        <v>26.707999999999899</v>
+        <v>27.9469999999999</v>
       </c>
       <c r="G3" t="s">
         <v>18</v>
       </c>
+      <c r="H3">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="I3">
+        <v>32.42</v>
+      </c>
       <c r="J3">
-        <v>1.54</v>
+        <v>1.31</v>
       </c>
       <c r="K3">
-        <v>41.13</v>
+        <v>36.61</v>
       </c>
       <c r="L3" t="s">
-        <v>630</v>
+        <v>642</v>
       </c>
       <c r="M3">
         <v>0</v>
@@ -14223,69 +13911,81 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>202</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s">
-        <v>625</v>
+        <v>640</v>
       </c>
       <c r="D4" t="s">
-        <v>626</v>
+        <v>641</v>
       </c>
       <c r="E4" t="s">
-        <v>240</v>
+        <v>45</v>
       </c>
       <c r="F4">
-        <v>24.859000000000002</v>
+        <v>36.610999999999898</v>
       </c>
       <c r="G4" t="s">
         <v>18</v>
       </c>
+      <c r="H4">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="I4">
+        <v>42.47</v>
+      </c>
       <c r="J4">
-        <v>1.56</v>
+        <v>1.31</v>
       </c>
       <c r="K4">
-        <v>38.78</v>
+        <v>47.96</v>
       </c>
       <c r="L4" t="s">
-        <v>631</v>
+        <v>643</v>
       </c>
       <c r="M4">
-        <v>15913</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>343</v>
       </c>
       <c r="B5" t="s">
-        <v>432</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
       <c r="D5" t="s">
-        <v>633</v>
+        <v>641</v>
       </c>
       <c r="E5" t="s">
         <v>45</v>
       </c>
       <c r="F5">
-        <v>41.091000000000001</v>
+        <v>39.006999999999898</v>
       </c>
       <c r="G5" t="s">
         <v>18</v>
       </c>
+      <c r="H5">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="I5">
+        <v>45.25</v>
+      </c>
       <c r="J5">
-        <v>1.32</v>
+        <v>1.36</v>
       </c>
       <c r="K5">
-        <v>54.24</v>
+        <v>53.05</v>
       </c>
       <c r="L5" t="s">
-        <v>616</v>
+        <v>644</v>
       </c>
       <c r="M5">
         <v>0</v>
@@ -14293,69 +13993,81 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>177</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>436</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s">
-        <v>625</v>
+        <v>640</v>
       </c>
       <c r="D6" t="s">
-        <v>626</v>
+        <v>641</v>
       </c>
       <c r="E6" t="s">
         <v>45</v>
       </c>
       <c r="F6">
-        <v>37.563000000000002</v>
+        <v>40.317</v>
       </c>
       <c r="G6" t="s">
         <v>18</v>
       </c>
+      <c r="H6">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="I6">
+        <v>46.77</v>
+      </c>
       <c r="J6">
-        <v>1.35</v>
+        <v>1.39</v>
       </c>
       <c r="K6">
-        <v>50.71</v>
+        <v>56.04</v>
       </c>
       <c r="L6" t="s">
-        <v>448</v>
+        <v>645</v>
       </c>
       <c r="M6">
-        <v>16287</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>380</v>
+        <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>628</v>
+        <v>646</v>
       </c>
       <c r="D7" t="s">
-        <v>629</v>
+        <v>647</v>
       </c>
       <c r="E7" t="s">
-        <v>240</v>
+        <v>45</v>
       </c>
       <c r="F7">
-        <v>26.739000000000001</v>
+        <v>30.34</v>
       </c>
       <c r="G7" t="s">
         <v>18</v>
       </c>
+      <c r="H7">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="I7">
+        <v>35.19</v>
+      </c>
       <c r="J7">
-        <v>1.61</v>
+        <v>1.41</v>
       </c>
       <c r="K7">
-        <v>43.05</v>
+        <v>42.78</v>
       </c>
       <c r="L7" t="s">
-        <v>634</v>
+        <v>648</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -14366,66 +14078,78 @@
         <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>252</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>625</v>
+        <v>649</v>
       </c>
       <c r="D8" t="s">
-        <v>626</v>
+        <v>650</v>
       </c>
       <c r="E8" t="s">
-        <v>240</v>
+        <v>17</v>
       </c>
       <c r="F8">
-        <v>28.117999999999899</v>
+        <v>68.076999999999899</v>
       </c>
       <c r="G8" t="s">
         <v>18</v>
       </c>
+      <c r="H8">
+        <v>1.21</v>
+      </c>
+      <c r="I8">
+        <v>82.37</v>
+      </c>
       <c r="J8">
-        <v>1.69</v>
+        <v>1.56</v>
       </c>
       <c r="K8">
-        <v>47.52</v>
+        <v>106.2</v>
       </c>
       <c r="L8" t="s">
-        <v>108</v>
+        <v>599</v>
       </c>
       <c r="M8">
-        <v>16883</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
       <c r="D9" t="s">
-        <v>633</v>
+        <v>641</v>
       </c>
       <c r="E9" t="s">
         <v>45</v>
       </c>
       <c r="F9">
-        <v>43.542000000000002</v>
+        <v>33.427999999999898</v>
       </c>
       <c r="G9" t="s">
         <v>18</v>
       </c>
+      <c r="H9">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="I9">
+        <v>38.78</v>
+      </c>
       <c r="J9">
-        <v>1.42</v>
+        <v>1.45</v>
       </c>
       <c r="K9">
-        <v>61.83</v>
+        <v>48.47</v>
       </c>
       <c r="L9" t="s">
-        <v>267</v>
+        <v>651</v>
       </c>
       <c r="M9">
         <v>0</v>
@@ -14433,107 +14157,43 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>135</v>
       </c>
       <c r="B10" t="s">
-        <v>208</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>625</v>
+        <v>640</v>
       </c>
       <c r="D10" t="s">
-        <v>626</v>
+        <v>641</v>
       </c>
       <c r="E10" t="s">
-        <v>240</v>
+        <v>45</v>
       </c>
       <c r="F10">
-        <v>31.337</v>
+        <v>38.040999999999897</v>
       </c>
       <c r="G10" t="s">
         <v>18</v>
       </c>
+      <c r="H10">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="I10">
+        <v>44.13</v>
+      </c>
       <c r="J10">
-        <v>1.69</v>
+        <v>1.46</v>
       </c>
       <c r="K10">
-        <v>52.96</v>
+        <v>55.54</v>
       </c>
       <c r="L10" t="s">
-        <v>635</v>
+        <v>532</v>
       </c>
       <c r="M10">
-        <v>16562</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>84</v>
-      </c>
-      <c r="B11" t="s">
-        <v>432</v>
-      </c>
-      <c r="C11" t="s">
-        <v>628</v>
-      </c>
-      <c r="D11" t="s">
-        <v>629</v>
-      </c>
-      <c r="E11" t="s">
-        <v>240</v>
-      </c>
-      <c r="F11">
-        <v>28.210999999999899</v>
-      </c>
-      <c r="G11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J11">
-        <v>1.71</v>
-      </c>
-      <c r="K11">
-        <v>48.24</v>
-      </c>
-      <c r="L11" t="s">
-        <v>547</v>
-      </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>315</v>
-      </c>
-      <c r="B12" t="s">
-        <v>410</v>
-      </c>
-      <c r="C12" t="s">
-        <v>625</v>
-      </c>
-      <c r="D12" t="s">
-        <v>626</v>
-      </c>
-      <c r="E12" t="s">
-        <v>240</v>
-      </c>
-      <c r="F12">
-        <v>26.491</v>
-      </c>
-      <c r="G12" t="s">
-        <v>18</v>
-      </c>
-      <c r="J12">
-        <v>1.73</v>
-      </c>
-      <c r="K12">
-        <v>45.83</v>
-      </c>
-      <c r="L12" t="s">
-        <v>636</v>
-      </c>
-      <c r="M12">
-        <v>17100</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -14542,9 +14202,13 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
-  <dimension ref="A1:M10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
+  <dimension ref="A1:M19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -14589,22 +14253,22 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>432</v>
       </c>
       <c r="C2" t="s">
-        <v>637</v>
+        <v>602</v>
       </c>
       <c r="D2" t="s">
-        <v>638</v>
+        <v>603</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
       </c>
       <c r="F2">
-        <v>62.2349999999999</v>
+        <v>42.976999999999897</v>
       </c>
       <c r="G2" t="s">
         <v>18</v>
@@ -14613,16 +14277,16 @@
         <v>1.21</v>
       </c>
       <c r="I2">
-        <v>75.3</v>
+        <v>52</v>
       </c>
       <c r="J2">
-        <v>1.32</v>
+        <v>1.31</v>
       </c>
       <c r="K2">
-        <v>82.15</v>
+        <v>56.3</v>
       </c>
       <c r="L2" t="s">
-        <v>639</v>
+        <v>604</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -14630,81 +14294,81 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="C3" t="s">
-        <v>640</v>
+        <v>605</v>
       </c>
       <c r="D3" t="s">
-        <v>641</v>
+        <v>606</v>
       </c>
       <c r="E3" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F3">
-        <v>27.9469999999999</v>
+        <v>40.137</v>
       </c>
       <c r="G3" t="s">
         <v>18</v>
       </c>
       <c r="H3">
-        <v>1.1599999999999999</v>
+        <v>1.21</v>
       </c>
       <c r="I3">
-        <v>32.42</v>
+        <v>48.57</v>
       </c>
       <c r="J3">
         <v>1.31</v>
       </c>
       <c r="K3">
-        <v>36.61</v>
+        <v>52.58</v>
       </c>
       <c r="L3" t="s">
-        <v>642</v>
+        <v>607</v>
       </c>
       <c r="M3">
-        <v>0</v>
+        <v>316540</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>104</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="C4" t="s">
-        <v>640</v>
+        <v>608</v>
       </c>
       <c r="D4" t="s">
-        <v>641</v>
+        <v>609</v>
       </c>
       <c r="E4" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F4">
-        <v>36.610999999999898</v>
+        <v>49.811999999999898</v>
       </c>
       <c r="G4" t="s">
         <v>18</v>
       </c>
       <c r="H4">
-        <v>1.1599999999999999</v>
+        <v>1.23</v>
       </c>
       <c r="I4">
-        <v>42.47</v>
+        <v>61.27</v>
       </c>
       <c r="J4">
-        <v>1.31</v>
+        <v>1.33</v>
       </c>
       <c r="K4">
-        <v>47.96</v>
+        <v>66.25</v>
       </c>
       <c r="L4" t="s">
-        <v>643</v>
+        <v>610</v>
       </c>
       <c r="M4">
         <v>0</v>
@@ -14712,81 +14376,75 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>343</v>
+        <v>109</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>380</v>
       </c>
       <c r="C5" t="s">
-        <v>640</v>
+        <v>605</v>
       </c>
       <c r="D5" t="s">
-        <v>641</v>
+        <v>606</v>
       </c>
       <c r="E5" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F5">
-        <v>39.006999999999898</v>
+        <v>54.6099999999999</v>
       </c>
       <c r="G5" t="s">
         <v>18</v>
       </c>
       <c r="H5">
-        <v>1.1599999999999999</v>
+        <v>1.25</v>
       </c>
       <c r="I5">
-        <v>45.25</v>
+        <v>68.260000000000005</v>
       </c>
       <c r="J5">
-        <v>1.36</v>
+        <v>1.41</v>
       </c>
       <c r="K5">
-        <v>53.05</v>
+        <v>77</v>
       </c>
       <c r="L5" t="s">
-        <v>644</v>
+        <v>611</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>316950</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>640</v>
+        <v>608</v>
       </c>
       <c r="D6" t="s">
-        <v>641</v>
+        <v>609</v>
       </c>
       <c r="E6" t="s">
-        <v>45</v>
+        <v>179</v>
       </c>
       <c r="F6">
-        <v>40.317</v>
+        <v>48.088999999999899</v>
       </c>
       <c r="G6" t="s">
         <v>18</v>
       </c>
-      <c r="H6">
-        <v>1.1599999999999999</v>
-      </c>
-      <c r="I6">
-        <v>46.77</v>
-      </c>
       <c r="J6">
-        <v>1.39</v>
+        <v>1.68</v>
       </c>
       <c r="K6">
-        <v>56.04</v>
+        <v>80.790000000000006</v>
       </c>
       <c r="L6" t="s">
-        <v>645</v>
+        <v>128</v>
       </c>
       <c r="M6">
         <v>0</v>
@@ -14794,40 +14452,40 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>646</v>
+        <v>612</v>
       </c>
       <c r="D7" t="s">
-        <v>647</v>
+        <v>613</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F7">
-        <v>30.34</v>
+        <v>33.817999999999898</v>
       </c>
       <c r="G7" t="s">
         <v>18</v>
       </c>
       <c r="H7">
-        <v>1.1599999999999999</v>
+        <v>1.25</v>
       </c>
       <c r="I7">
-        <v>35.19</v>
+        <v>42.27</v>
       </c>
       <c r="J7">
-        <v>1.41</v>
+        <v>1.43</v>
       </c>
       <c r="K7">
-        <v>42.78</v>
+        <v>48.36</v>
       </c>
       <c r="L7" t="s">
-        <v>648</v>
+        <v>614</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -14835,125 +14493,494 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>380</v>
       </c>
       <c r="C8" t="s">
-        <v>649</v>
+        <v>605</v>
       </c>
       <c r="D8" t="s">
-        <v>650</v>
+        <v>606</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
       </c>
       <c r="F8">
-        <v>68.076999999999899</v>
+        <v>20.4149999999999</v>
       </c>
       <c r="G8" t="s">
         <v>18</v>
       </c>
       <c r="H8">
-        <v>1.21</v>
+        <v>1.42</v>
       </c>
       <c r="I8">
-        <v>82.37</v>
+        <v>28.99</v>
       </c>
       <c r="J8">
-        <v>1.56</v>
+        <v>1.47</v>
       </c>
       <c r="K8">
-        <v>106.2</v>
+        <v>30.01</v>
       </c>
       <c r="L8" t="s">
-        <v>599</v>
+        <v>615</v>
       </c>
       <c r="M8">
-        <v>0</v>
+        <v>317270</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>274</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="C9" t="s">
-        <v>640</v>
+        <v>602</v>
       </c>
       <c r="D9" t="s">
-        <v>641</v>
+        <v>603</v>
       </c>
       <c r="E9" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F9">
-        <v>33.427999999999898</v>
+        <v>36.362000000000002</v>
       </c>
       <c r="G9" t="s">
         <v>18</v>
       </c>
       <c r="H9">
-        <v>1.1599999999999999</v>
+        <v>1.46</v>
       </c>
       <c r="I9">
-        <v>38.78</v>
+        <v>53.09</v>
       </c>
       <c r="J9">
-        <v>1.45</v>
+        <v>1.52</v>
       </c>
       <c r="K9">
-        <v>48.47</v>
+        <v>55.27</v>
       </c>
       <c r="L9" t="s">
-        <v>651</v>
+        <v>616</v>
       </c>
       <c r="M9">
-        <v>0</v>
+        <v>430120</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>274</v>
+      </c>
+      <c r="B10" t="s">
+        <v>380</v>
+      </c>
+      <c r="C10" t="s">
+        <v>605</v>
+      </c>
+      <c r="D10" t="s">
+        <v>606</v>
+      </c>
+      <c r="E10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10">
+        <v>30.867999999999899</v>
+      </c>
+      <c r="G10" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10">
+        <v>1.46</v>
+      </c>
+      <c r="I10">
+        <v>45.07</v>
+      </c>
+      <c r="J10">
+        <v>1.51</v>
+      </c>
+      <c r="K10">
+        <v>46.61</v>
+      </c>
+      <c r="L10" t="s">
+        <v>617</v>
+      </c>
+      <c r="M10">
+        <v>317370</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>612</v>
+      </c>
+      <c r="D11" t="s">
+        <v>613</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11">
+        <v>24.591999999999899</v>
+      </c>
+      <c r="G11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H11">
+        <v>1.46</v>
+      </c>
+      <c r="I11">
+        <v>35.9</v>
+      </c>
+      <c r="J11">
+        <v>1.52</v>
+      </c>
+      <c r="K11">
+        <v>37.380000000000003</v>
+      </c>
+      <c r="L11" t="s">
+        <v>618</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" t="s">
+        <v>380</v>
+      </c>
+      <c r="C12" t="s">
+        <v>605</v>
+      </c>
+      <c r="D12" t="s">
+        <v>606</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12">
+        <v>22.882000000000001</v>
+      </c>
+      <c r="G12" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12">
+        <v>1.48</v>
+      </c>
+      <c r="I12">
+        <v>33.869999999999997</v>
+      </c>
+      <c r="J12">
+        <v>1.53</v>
+      </c>
+      <c r="K12">
+        <v>35.01</v>
+      </c>
+      <c r="L12" t="s">
+        <v>619</v>
+      </c>
+      <c r="M12">
+        <v>317685</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>299</v>
+      </c>
+      <c r="B13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" t="s">
+        <v>605</v>
+      </c>
+      <c r="D13" t="s">
+        <v>606</v>
+      </c>
+      <c r="E13" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13">
+        <v>44.963000000000001</v>
+      </c>
+      <c r="G13" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13">
+        <v>1.54</v>
+      </c>
+      <c r="I13">
+        <v>69.239999999999995</v>
+      </c>
+      <c r="J13">
+        <v>1.6</v>
+      </c>
+      <c r="K13">
+        <v>71.94</v>
+      </c>
+      <c r="L13" t="s">
+        <v>505</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>299</v>
+      </c>
+      <c r="B14" t="s">
+        <v>224</v>
+      </c>
+      <c r="C14" t="s">
+        <v>605</v>
+      </c>
+      <c r="D14" t="s">
+        <v>606</v>
+      </c>
+      <c r="E14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14">
+        <v>30.207999999999899</v>
+      </c>
+      <c r="G14" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14">
+        <v>1.54</v>
+      </c>
+      <c r="I14">
+        <v>46.52</v>
+      </c>
+      <c r="J14">
+        <v>1.59</v>
+      </c>
+      <c r="K14">
+        <v>48.03</v>
+      </c>
+      <c r="L14" t="s">
+        <v>620</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B15" t="s">
+        <v>93</v>
+      </c>
+      <c r="C15" t="s">
+        <v>608</v>
+      </c>
+      <c r="D15" t="s">
+        <v>609</v>
+      </c>
+      <c r="E15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15">
+        <v>48.701999999999899</v>
+      </c>
+      <c r="G15" t="s">
+        <v>18</v>
+      </c>
+      <c r="H15">
+        <v>1.6</v>
+      </c>
+      <c r="I15">
+        <v>77.92</v>
+      </c>
+      <c r="J15">
+        <v>1.61</v>
+      </c>
+      <c r="K15">
+        <v>78.41</v>
+      </c>
+      <c r="L15" t="s">
+        <v>130</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>69</v>
+      </c>
+      <c r="B16" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" t="s">
+        <v>612</v>
+      </c>
+      <c r="D16" t="s">
+        <v>613</v>
+      </c>
+      <c r="E16" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16">
+        <v>32.783000000000001</v>
+      </c>
+      <c r="G16" t="s">
+        <v>18</v>
+      </c>
+      <c r="H16">
+        <v>1.6</v>
+      </c>
+      <c r="I16">
+        <v>52.45</v>
+      </c>
+      <c r="J16">
+        <v>1.61</v>
+      </c>
+      <c r="K16">
+        <v>52.78</v>
+      </c>
+      <c r="L16" t="s">
+        <v>621</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" t="s">
+        <v>602</v>
+      </c>
+      <c r="D17" t="s">
+        <v>603</v>
+      </c>
+      <c r="E17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17">
+        <v>40.512</v>
+      </c>
+      <c r="G17" t="s">
+        <v>18</v>
+      </c>
+      <c r="H17">
+        <v>1.6</v>
+      </c>
+      <c r="I17">
+        <v>64.819999999999993</v>
+      </c>
+      <c r="J17">
+        <v>1.62</v>
+      </c>
+      <c r="K17">
+        <v>65.63</v>
+      </c>
+      <c r="L17" t="s">
+        <v>622</v>
+      </c>
+      <c r="M17">
+        <v>430652</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>135</v>
       </c>
-      <c r="B10" t="s">
-        <v>70</v>
-      </c>
-      <c r="C10" t="s">
-        <v>640</v>
-      </c>
-      <c r="D10" t="s">
-        <v>641</v>
-      </c>
-      <c r="E10" t="s">
-        <v>45</v>
-      </c>
-      <c r="F10">
-        <v>38.040999999999897</v>
-      </c>
-      <c r="G10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10">
-        <v>1.1599999999999999</v>
-      </c>
-      <c r="I10">
-        <v>44.13</v>
-      </c>
-      <c r="J10">
-        <v>1.46</v>
-      </c>
-      <c r="K10">
-        <v>55.54</v>
-      </c>
-      <c r="L10" t="s">
-        <v>532</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
+      <c r="B18" t="s">
+        <v>224</v>
+      </c>
+      <c r="C18" t="s">
+        <v>605</v>
+      </c>
+      <c r="D18" t="s">
+        <v>606</v>
+      </c>
+      <c r="E18" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18">
+        <v>28.27</v>
+      </c>
+      <c r="G18" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18">
+        <v>1.61</v>
+      </c>
+      <c r="I18">
+        <v>45.51</v>
+      </c>
+      <c r="J18">
+        <v>1.63</v>
+      </c>
+      <c r="K18">
+        <v>46.08</v>
+      </c>
+      <c r="L18" t="s">
+        <v>623</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" t="s">
+        <v>380</v>
+      </c>
+      <c r="C19" t="s">
+        <v>605</v>
+      </c>
+      <c r="D19" t="s">
+        <v>606</v>
+      </c>
+      <c r="E19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19">
+        <v>50.142000000000003</v>
+      </c>
+      <c r="G19" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19">
+        <v>1.64</v>
+      </c>
+      <c r="I19">
+        <v>82.23</v>
+      </c>
+      <c r="J19">
+        <v>1.69</v>
+      </c>
+      <c r="K19">
+        <v>84.74</v>
+      </c>
+      <c r="L19" t="s">
+        <v>624</v>
+      </c>
+      <c r="M19">
+        <v>318930</v>
       </c>
     </row>
   </sheetData>
@@ -14965,6 +14992,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -28863,6 +28895,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <dimension ref="A1:M103"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="9" max="9" width="16.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
UPDATE: calculation for profit
</commit_message>
<xml_diff>
--- a/A_FINAL_RESULT/eko_transactions.xlsx
+++ b/A_FINAL_RESULT/eko_transactions.xlsx
@@ -568,10 +568,10 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>1.69</v>
+        <v>1.65</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -580,7 +580,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>138.58</v>
+        <v>135.3</v>
       </c>
       <c r="M2" t="n">
         <v>1.69</v>
@@ -628,10 +628,10 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>1.69</v>
+        <v>1.65</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -640,7 +640,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>28.04</v>
+        <v>27.38</v>
       </c>
       <c r="M3" t="n">
         <v>1.69</v>
@@ -688,19 +688,19 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>1.7</v>
+        <v>1.66</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>0.26</v>
       </c>
       <c r="L4" t="n">
-        <v>43.44</v>
+        <v>42.42</v>
       </c>
       <c r="M4" t="n">
         <v>1.7</v>
@@ -748,19 +748,19 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>1.72</v>
+        <v>1.68</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="L5" t="n">
-        <v>39.99</v>
+        <v>39.06</v>
       </c>
       <c r="M5" t="n">
         <v>1.72</v>
@@ -808,19 +808,19 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>1.76</v>
+        <v>1.72</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>-0.26</v>
       </c>
       <c r="L6" t="n">
-        <v>46.46</v>
+        <v>45.4</v>
       </c>
       <c r="M6" t="n">
         <v>1.76</v>
@@ -876,9 +876,7 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>100.56</v>
       </c>
@@ -928,19 +926,19 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>1.71</v>
+        <v>1.73</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>4.2</v>
+        <v>1.4</v>
       </c>
       <c r="L8" t="n">
-        <v>119.72</v>
+        <v>121.12</v>
       </c>
       <c r="M8" t="n">
         <v>1.77</v>
@@ -1093,7 +1091,7 @@
         <v>0.03</v>
       </c>
       <c r="K2" t="n">
-        <v>2.32</v>
+        <v>0.87</v>
       </c>
       <c r="L2" t="n">
         <v>41.49</v>
@@ -1153,7 +1151,7 @@
         <v>0.03</v>
       </c>
       <c r="K3" t="n">
-        <v>1.27</v>
+        <v>0.48</v>
       </c>
       <c r="L3" t="n">
         <v>22.74</v>
@@ -1213,7 +1211,7 @@
         <v>0.03</v>
       </c>
       <c r="K4" t="n">
-        <v>1.54</v>
+        <v>0.66</v>
       </c>
       <c r="L4" t="n">
         <v>31.45</v>
@@ -1273,7 +1271,7 @@
         <v>0.03</v>
       </c>
       <c r="K5" t="n">
-        <v>0.88</v>
+        <v>0.38</v>
       </c>
       <c r="L5" t="n">
         <v>18.15</v>
@@ -1333,7 +1331,7 @@
         <v>0.03</v>
       </c>
       <c r="K6" t="n">
-        <v>1.82</v>
+        <v>0.68</v>
       </c>
       <c r="L6" t="n">
         <v>32.82</v>
@@ -1489,7 +1487,7 @@
         <v>0.09</v>
       </c>
       <c r="K2" t="n">
-        <v>13.86</v>
+        <v>5.94</v>
       </c>
       <c r="L2" t="n">
         <v>119.46</v>
@@ -1644,9 +1642,7 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>42.23</v>
       </c>
@@ -1704,9 +1700,7 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>57.8</v>
       </c>
@@ -1764,9 +1758,7 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>22.39</v>
       </c>
@@ -1824,9 +1816,7 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>62.81</v>
       </c>
@@ -1884,9 +1874,7 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>34.31</v>
       </c>
@@ -1944,9 +1932,7 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>28.62</v>
       </c>
@@ -2004,9 +1990,7 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>68.18000000000001</v>
       </c>
@@ -2064,9 +2048,7 @@
       <c r="J9" t="n">
         <v>0</v>
       </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>29.6</v>
       </c>
@@ -2125,7 +2107,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>1.96</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
         <v>84.09</v>
@@ -2185,7 +2167,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>1.74</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>74.7</v>
@@ -2245,7 +2227,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0.93</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
         <v>40.04</v>
@@ -2305,7 +2287,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>2.68</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>76.26000000000001</v>
@@ -2364,9 +2346,7 @@
       <c r="J14" t="n">
         <v>0</v>
       </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>30.33</v>
       </c>
@@ -2425,7 +2405,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>39.64</v>
@@ -2484,9 +2464,7 @@
       <c r="J16" t="n">
         <v>0</v>
       </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
         <v>4.34</v>
       </c>
@@ -2545,7 +2523,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>2.78</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>35.42</v>
@@ -2605,7 +2583,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>14.34</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>86.56</v>
@@ -2664,9 +2642,7 @@
       <c r="J19" t="n">
         <v>0</v>
       </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="n">
         <v>10.82</v>
       </c>
@@ -2725,7 +2701,7 @@
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>3.13</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>90.7</v>
@@ -2785,7 +2761,7 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>3.33</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
         <v>82.83</v>
@@ -2941,7 +2917,7 @@
         <v>0.01</v>
       </c>
       <c r="K2" t="n">
-        <v>14.1</v>
+        <v>4.7</v>
       </c>
       <c r="L2" t="n">
         <v>780.2</v>
@@ -3001,7 +2977,7 @@
         <v>0.01</v>
       </c>
       <c r="K3" t="n">
-        <v>22.67</v>
+        <v>3.78</v>
       </c>
       <c r="L3" t="n">
         <v>627.2</v>
@@ -3181,7 +3157,7 @@
         <v>0.02</v>
       </c>
       <c r="K6" t="n">
-        <v>14.4</v>
+        <v>7.2</v>
       </c>
       <c r="L6" t="n">
         <v>622.84</v>
@@ -3241,7 +3217,7 @@
         <v>0.02</v>
       </c>
       <c r="K7" t="n">
-        <v>3.31</v>
+        <v>1.1</v>
       </c>
       <c r="L7" t="n">
         <v>95.52</v>
@@ -3301,7 +3277,7 @@
         <v>0.02</v>
       </c>
       <c r="K8" t="n">
-        <v>13.42</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="L8" t="n">
         <v>787.34</v>
@@ -3361,7 +3337,7 @@
         <v>0.02</v>
       </c>
       <c r="K9" t="n">
-        <v>11.51</v>
+        <v>7.68</v>
       </c>
       <c r="L9" t="n">
         <v>675.49</v>
@@ -3516,9 +3492,7 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>55.7</v>
       </c>
@@ -3576,9 +3550,7 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>13.28</v>
       </c>
@@ -3636,9 +3608,7 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>128.74</v>
       </c>
@@ -3696,9 +3666,7 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>23.79</v>
       </c>
@@ -3756,9 +3724,7 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>9.49</v>
       </c>
@@ -3816,9 +3782,7 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>138.34</v>
       </c>
@@ -3876,9 +3840,7 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>9.49</v>
       </c>
@@ -3936,9 +3898,7 @@
       <c r="J9" t="n">
         <v>0</v>
       </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>118.94</v>
       </c>
@@ -3996,9 +3956,7 @@
       <c r="J10" t="n">
         <v>0</v>
       </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
         <v>77.45999999999999</v>
       </c>
@@ -4056,9 +4014,7 @@
       <c r="J11" t="n">
         <v>0</v>
       </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>118.61</v>
       </c>
@@ -4116,9 +4072,7 @@
       <c r="J12" t="n">
         <v>0</v>
       </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
         <v>78.26000000000001</v>
       </c>
@@ -4273,7 +4227,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.57</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>37.03</v>
@@ -4333,7 +4287,7 @@
         <v>0.03</v>
       </c>
       <c r="K3" t="n">
-        <v>3.66</v>
+        <v>1.57</v>
       </c>
       <c r="L3" t="n">
         <v>74.67</v>
@@ -4393,7 +4347,7 @@
         <v>0.03</v>
       </c>
       <c r="K4" t="n">
-        <v>2.25</v>
+        <v>0.75</v>
       </c>
       <c r="L4" t="n">
         <v>35.78</v>
@@ -4453,7 +4407,7 @@
         <v>0.03</v>
       </c>
       <c r="K5" t="n">
-        <v>1.67</v>
+        <v>0.55</v>
       </c>
       <c r="L5" t="n">
         <v>26.46</v>
@@ -4513,7 +4467,7 @@
         <v>0.03</v>
       </c>
       <c r="K6" t="n">
-        <v>2.01</v>
+        <v>0.86</v>
       </c>
       <c r="L6" t="n">
         <v>41.33</v>
@@ -4669,7 +4623,7 @@
         <v>0.01</v>
       </c>
       <c r="K2" t="n">
-        <v>3.16</v>
+        <v>0.45</v>
       </c>
       <c r="L2" t="n">
         <v>76.37</v>
@@ -4729,7 +4683,7 @@
         <v>0.01</v>
       </c>
       <c r="K3" t="n">
-        <v>10.78</v>
+        <v>1.54</v>
       </c>
       <c r="L3" t="n">
         <v>260.37</v>
@@ -4789,7 +4743,7 @@
         <v>0.01</v>
       </c>
       <c r="K4" t="n">
-        <v>3.36</v>
+        <v>0.48</v>
       </c>
       <c r="L4" t="n">
         <v>81.12</v>
@@ -4849,7 +4803,7 @@
         <v>0.01</v>
       </c>
       <c r="K5" t="n">
-        <v>3.78</v>
+        <v>0.54</v>
       </c>
       <c r="L5" t="n">
         <v>91.26000000000001</v>
@@ -5005,7 +4959,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>20.51</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>676.75</v>
@@ -5065,7 +5019,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>36.05</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>849.8</v>
@@ -5125,7 +5079,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>27.24</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>641.98</v>
@@ -5185,7 +5139,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>47.6</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>1122.05</v>
@@ -5245,7 +5199,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>660.02</v>
@@ -5400,9 +5354,7 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>341.72</v>
       </c>
@@ -5460,9 +5412,7 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>340.02</v>
       </c>
@@ -5520,9 +5470,7 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>173</v>
       </c>
@@ -5580,9 +5528,7 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>256.66</v>
       </c>
@@ -5641,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>215.07</v>
@@ -5701,7 +5647,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>8.43</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>362.58</v>
@@ -5761,7 +5707,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>7.21</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
         <v>248.09</v>
@@ -5821,7 +5767,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>12.36</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
         <v>352.26</v>
@@ -5881,7 +5827,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>13.2</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
         <v>376.2</v>
@@ -5941,7 +5887,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>10.2</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>295.8</v>
@@ -6001,7 +5947,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>6.9</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
         <v>200.1</v>
@@ -6156,9 +6102,7 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>96.98</v>
       </c>
@@ -6373,7 +6317,7 @@
         <v>0.04</v>
       </c>
       <c r="K3" t="n">
-        <v>4.83</v>
+        <v>3.22</v>
       </c>
       <c r="L3" t="n">
         <v>116.02</v>
@@ -6529,7 +6473,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.13</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>37.26</v>
@@ -6589,7 +6533,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1.03</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>33.99</v>
@@ -6649,7 +6593,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>2.88</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>67.92</v>
@@ -6709,7 +6653,7 @@
         <v>0.01</v>
       </c>
       <c r="K5" t="n">
-        <v>1.3</v>
+        <v>0.43</v>
       </c>
       <c r="L5" t="n">
         <v>74.91</v>
@@ -6769,7 +6713,7 @@
         <v>0.02</v>
       </c>
       <c r="K6" t="n">
-        <v>0.92</v>
+        <v>0.46</v>
       </c>
       <c r="L6" t="n">
         <v>39.68</v>
@@ -6829,7 +6773,7 @@
         <v>0.02</v>
       </c>
       <c r="K7" t="n">
-        <v>1.36</v>
+        <v>0.91</v>
       </c>
       <c r="L7" t="n">
         <v>79.65000000000001</v>
@@ -6889,7 +6833,7 @@
         <v>0.02</v>
       </c>
       <c r="K8" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="L8" t="n">
         <v>96.93000000000001</v>
@@ -7044,9 +6988,7 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>60.17</v>
       </c>
@@ -7104,9 +7046,7 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>4.34</v>
       </c>
@@ -7164,9 +7104,7 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>49.21</v>
       </c>
@@ -7224,9 +7162,7 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>63.15</v>
       </c>
@@ -7284,9 +7220,7 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>69.91</v>
       </c>
@@ -7440,9 +7374,7 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>51.83</v>
       </c>
@@ -7500,9 +7432,7 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>18.4</v>
       </c>
@@ -7561,7 +7491,7 @@
         <v>0.03</v>
       </c>
       <c r="K4" t="n">
-        <v>2.09</v>
+        <v>0.89</v>
       </c>
       <c r="L4" t="n">
         <v>42.66</v>
@@ -7621,7 +7551,7 @@
         <v>0.03</v>
       </c>
       <c r="K5" t="n">
-        <v>1.39</v>
+        <v>0.52</v>
       </c>
       <c r="L5" t="n">
         <v>24.85</v>
@@ -7681,7 +7611,7 @@
         <v>0.03</v>
       </c>
       <c r="K6" t="n">
-        <v>2.48</v>
+        <v>1.06</v>
       </c>
       <c r="L6" t="n">
         <v>50.94</v>
@@ -7837,7 +7767,7 @@
         <v>0.03</v>
       </c>
       <c r="K2" t="n">
-        <v>1.98</v>
+        <v>1.19</v>
       </c>
       <c r="L2" t="n">
         <v>56.76</v>
@@ -7897,7 +7827,7 @@
         <v>0.01</v>
       </c>
       <c r="K3" t="n">
-        <v>1.93</v>
+        <v>0.48</v>
       </c>
       <c r="L3" t="n">
         <v>83.53</v>
@@ -8053,7 +7983,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>2.44</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>80.62</v>
@@ -8113,7 +8043,7 @@
         <v>0.01</v>
       </c>
       <c r="K3" t="n">
-        <v>2.11</v>
+        <v>0.7</v>
       </c>
       <c r="L3" t="n">
         <v>121.44</v>
@@ -8269,7 +8199,7 @@
         <v>0.01</v>
       </c>
       <c r="K2" t="n">
-        <v>1.03</v>
+        <v>0.34</v>
       </c>
       <c r="L2" t="n">
         <v>59.25</v>
@@ -8425,7 +8355,7 @@
         <v>0.03</v>
       </c>
       <c r="K2" t="n">
-        <v>3.17</v>
+        <v>1.36</v>
       </c>
       <c r="L2" t="n">
         <v>64.81</v>
@@ -8485,7 +8415,7 @@
         <v>0.03</v>
       </c>
       <c r="K3" t="n">
-        <v>2.22</v>
+        <v>0.95</v>
       </c>
       <c r="L3" t="n">
         <v>45.68</v>
@@ -8544,9 +8474,7 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>4.34</v>
       </c>
@@ -8605,7 +8533,7 @@
         <v>0.03</v>
       </c>
       <c r="K5" t="n">
-        <v>3.84</v>
+        <v>1.65</v>
       </c>
       <c r="L5" t="n">
         <v>79.09</v>
@@ -8761,7 +8689,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>49.5</v>
@@ -8821,7 +8749,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>3.79</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>89.38</v>
@@ -8881,7 +8809,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1.57</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>32.41</v>
@@ -8941,7 +8869,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>10.01</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>235.95</v>
@@ -9001,7 +8929,7 @@
         <v>0.03</v>
       </c>
       <c r="K6" t="n">
-        <v>0.58</v>
+        <v>0.25</v>
       </c>
       <c r="L6" t="n">
         <v>11.85</v>
@@ -9061,7 +8989,7 @@
         <v>0.01</v>
       </c>
       <c r="K7" t="n">
-        <v>1.31</v>
+        <v>0.44</v>
       </c>
       <c r="L7" t="n">
         <v>75.5</v>
@@ -9121,7 +9049,7 @@
         <v>0.03</v>
       </c>
       <c r="K8" t="n">
-        <v>0.68</v>
+        <v>0.29</v>
       </c>
       <c r="L8" t="n">
         <v>13.85</v>
@@ -9181,7 +9109,7 @@
         <v>0.01</v>
       </c>
       <c r="K9" t="n">
-        <v>1.48</v>
+        <v>0.49</v>
       </c>
       <c r="L9" t="n">
         <v>85.29000000000001</v>
@@ -9241,7 +9169,7 @@
         <v>0.01</v>
       </c>
       <c r="K10" t="n">
-        <v>1.88</v>
+        <v>0.63</v>
       </c>
       <c r="L10" t="n">
         <v>108.56</v>
@@ -9301,7 +9229,7 @@
         <v>0.01</v>
       </c>
       <c r="K11" t="n">
-        <v>1.37</v>
+        <v>0.46</v>
       </c>
       <c r="L11" t="n">
         <v>79.03</v>
@@ -9361,7 +9289,7 @@
         <v>0.01</v>
       </c>
       <c r="K12" t="n">
-        <v>1.49</v>
+        <v>0.5</v>
       </c>
       <c r="L12" t="n">
         <v>85.79000000000001</v>
@@ -9420,9 +9348,7 @@
       <c r="J13" t="n">
         <v>0</v>
       </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
         <v>9.49</v>
       </c>
@@ -9481,7 +9407,7 @@
         <v>0.01</v>
       </c>
       <c r="K14" t="n">
-        <v>1.21</v>
+        <v>0.4</v>
       </c>
       <c r="L14" t="n">
         <v>69.79000000000001</v>
@@ -9541,7 +9467,7 @@
         <v>0.01</v>
       </c>
       <c r="K15" t="n">
-        <v>0.86</v>
+        <v>0.43</v>
       </c>
       <c r="L15" t="n">
         <v>74.39</v>
@@ -9601,7 +9527,7 @@
         <v>0.01</v>
       </c>
       <c r="K16" t="n">
-        <v>1.62</v>
+        <v>0.54</v>
       </c>
       <c r="L16" t="n">
         <v>93.68000000000001</v>
@@ -9661,7 +9587,7 @@
         <v>0.01</v>
       </c>
       <c r="K17" t="n">
-        <v>1.29</v>
+        <v>0.43</v>
       </c>
       <c r="L17" t="n">
         <v>74.39</v>
@@ -9721,7 +9647,7 @@
         <v>0.01</v>
       </c>
       <c r="K18" t="n">
-        <v>1.62</v>
+        <v>0.54</v>
       </c>
       <c r="L18" t="n">
         <v>93.42</v>
@@ -9781,7 +9707,7 @@
         <v>0.01</v>
       </c>
       <c r="K19" t="n">
-        <v>1.02</v>
+        <v>0.34</v>
       </c>
       <c r="L19" t="n">
         <v>58.78</v>
@@ -9841,7 +9767,7 @@
         <v>0.01</v>
       </c>
       <c r="K20" t="n">
-        <v>1.02</v>
+        <v>0.34</v>
       </c>
       <c r="L20" t="n">
         <v>58.82</v>
@@ -9901,7 +9827,7 @@
         <v>0.01</v>
       </c>
       <c r="K21" t="n">
-        <v>1.85</v>
+        <v>0.46</v>
       </c>
       <c r="L21" t="n">
         <v>79.87</v>
@@ -9961,7 +9887,7 @@
         <v>0.01</v>
       </c>
       <c r="K22" t="n">
-        <v>1.58</v>
+        <v>0.4</v>
       </c>
       <c r="L22" t="n">
         <v>68.34999999999999</v>
@@ -10021,7 +9947,7 @@
         <v>0.01</v>
       </c>
       <c r="K23" t="n">
-        <v>1.2</v>
+        <v>0.3</v>
       </c>
       <c r="L23" t="n">
         <v>51.9</v>
@@ -10081,7 +10007,7 @@
         <v>0.01</v>
       </c>
       <c r="K24" t="n">
-        <v>1.8</v>
+        <v>0.45</v>
       </c>
       <c r="L24" t="n">
         <v>77.84999999999999</v>
@@ -10141,7 +10067,7 @@
         <v>0.03</v>
       </c>
       <c r="K25" t="n">
-        <v>0.43</v>
+        <v>0.18</v>
       </c>
       <c r="L25" t="n">
         <v>8.69</v>
@@ -10201,7 +10127,7 @@
         <v>0.01</v>
       </c>
       <c r="K26" t="n">
-        <v>2.21</v>
+        <v>0.55</v>
       </c>
       <c r="L26" t="n">
         <v>95.53</v>
@@ -10261,7 +10187,7 @@
         <v>0.02</v>
       </c>
       <c r="K27" t="n">
-        <v>1.47</v>
+        <v>0.74</v>
       </c>
       <c r="L27" t="n">
         <v>63.65</v>
@@ -10321,7 +10247,7 @@
         <v>0.02</v>
       </c>
       <c r="K28" t="n">
-        <v>2.01</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
         <v>86.84</v>
@@ -10381,7 +10307,7 @@
         <v>0.02</v>
       </c>
       <c r="K29" t="n">
-        <v>2.37</v>
+        <v>1.19</v>
       </c>
       <c r="L29" t="n">
         <v>102.59</v>
@@ -10441,7 +10367,7 @@
         <v>0.02</v>
       </c>
       <c r="K30" t="n">
-        <v>1.93</v>
+        <v>0.96</v>
       </c>
       <c r="L30" t="n">
         <v>83.26000000000001</v>
@@ -10501,7 +10427,7 @@
         <v>0.02</v>
       </c>
       <c r="K31" t="n">
-        <v>1.42</v>
+        <v>0.71</v>
       </c>
       <c r="L31" t="n">
         <v>61.57</v>
@@ -10561,7 +10487,7 @@
         <v>0.02</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L32" t="n">
         <v>86.38</v>
@@ -10621,7 +10547,7 @@
         <v>0.02</v>
       </c>
       <c r="K33" t="n">
-        <v>1.62</v>
+        <v>1.08</v>
       </c>
       <c r="L33" t="n">
         <v>95.04000000000001</v>
@@ -10681,7 +10607,7 @@
         <v>0.03</v>
       </c>
       <c r="K34" t="n">
-        <v>0.6</v>
+        <v>0.26</v>
       </c>
       <c r="L34" t="n">
         <v>12.4</v>
@@ -10740,9 +10666,7 @@
       <c r="J35" t="n">
         <v>0</v>
       </c>
-      <c r="K35" t="n">
-        <v>0</v>
-      </c>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
         <v>49.08</v>
       </c>
@@ -10801,7 +10725,7 @@
         <v>0.02</v>
       </c>
       <c r="K36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L36" t="n">
         <v>88</v>
@@ -10861,7 +10785,7 @@
         <v>0.02</v>
       </c>
       <c r="K37" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="L37" t="n">
         <v>70.23999999999999</v>
@@ -10921,7 +10845,7 @@
         <v>0.02</v>
       </c>
       <c r="K38" t="n">
-        <v>2.11</v>
+        <v>1.06</v>
       </c>
       <c r="L38" t="n">
         <v>93.02</v>
@@ -10980,9 +10904,7 @@
       <c r="J39" t="n">
         <v>0</v>
       </c>
-      <c r="K39" t="n">
-        <v>0</v>
-      </c>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" t="n">
         <v>17.71</v>
       </c>
@@ -11137,7 +11059,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>2.48</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>58.53</v>
@@ -11197,7 +11119,7 @@
         <v>0.03</v>
       </c>
       <c r="K3" t="n">
-        <v>2.44</v>
+        <v>0.92</v>
       </c>
       <c r="L3" t="n">
         <v>43.62</v>
@@ -11257,7 +11179,7 @@
         <v>0.01</v>
       </c>
       <c r="K4" t="n">
-        <v>0.45</v>
+        <v>0.11</v>
       </c>
       <c r="L4" t="n">
         <v>19.55</v>
@@ -11317,7 +11239,7 @@
         <v>0.02</v>
       </c>
       <c r="K5" t="n">
-        <v>1.66</v>
+        <v>0.83</v>
       </c>
       <c r="L5" t="n">
         <v>71.73999999999999</v>
@@ -11377,7 +11299,7 @@
         <v>0.02</v>
       </c>
       <c r="K6" t="n">
-        <v>1.53</v>
+        <v>0.44</v>
       </c>
       <c r="L6" t="n">
         <v>37.94</v>
@@ -11437,7 +11359,7 @@
         <v>0.02</v>
       </c>
       <c r="K7" t="n">
-        <v>2.22</v>
+        <v>1.11</v>
       </c>
       <c r="L7" t="n">
         <v>97.79000000000001</v>
@@ -11497,7 +11419,7 @@
         <v>0.02</v>
       </c>
       <c r="K8" t="n">
-        <v>2.88</v>
+        <v>1.44</v>
       </c>
       <c r="L8" t="n">
         <v>126.72</v>
@@ -11557,7 +11479,7 @@
         <v>0.02</v>
       </c>
       <c r="K9" t="n">
-        <v>0.77</v>
+        <v>0.31</v>
       </c>
       <c r="L9" t="n">
         <v>27.25</v>
@@ -11712,9 +11634,7 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>57.46</v>
       </c>
@@ -11772,9 +11692,7 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>64.7</v>
       </c>
@@ -11832,9 +11750,7 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>96.34999999999999</v>
       </c>
@@ -11892,9 +11808,7 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>83.67</v>
       </c>
@@ -11952,9 +11866,7 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>91.53</v>
       </c>
@@ -12012,9 +11924,7 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>37.4</v>
       </c>
@@ -12072,9 +11982,7 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>41.54</v>
       </c>
@@ -12132,9 +12040,7 @@
       <c r="J9" t="n">
         <v>0</v>
       </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>43</v>
       </c>
@@ -12192,9 +12098,7 @@
       <c r="J10" t="n">
         <v>0</v>
       </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
         <v>80.65000000000001</v>
       </c>
@@ -12252,9 +12156,7 @@
       <c r="J11" t="n">
         <v>0</v>
       </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>29.92</v>
       </c>
@@ -12312,9 +12214,7 @@
       <c r="J12" t="n">
         <v>0</v>
       </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
         <v>57</v>
       </c>
@@ -12372,9 +12272,7 @@
       <c r="J13" t="n">
         <v>0</v>
       </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
         <v>42.01</v>
       </c>
@@ -12432,9 +12330,7 @@
       <c r="J14" t="n">
         <v>0</v>
       </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>109.12</v>
       </c>
@@ -12492,9 +12388,7 @@
       <c r="J15" t="n">
         <v>0</v>
       </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>45</v>
       </c>
@@ -12553,7 +12447,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>1.08</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>30.78</v>
@@ -12613,7 +12507,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>2.99</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>85.31999999999999</v>
@@ -12673,7 +12567,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>2.61</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>90.98999999999999</v>
@@ -12733,7 +12627,7 @@
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
         <v>43.71</v>
@@ -12793,7 +12687,7 @@
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>1.77</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>61.56</v>
@@ -12853,7 +12747,7 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
         <v>42.33</v>
@@ -12913,7 +12807,7 @@
         <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
         <v>87</v>
@@ -12973,7 +12867,7 @@
         <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
         <v>87</v>
@@ -13033,7 +12927,7 @@
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
         <v>69.59999999999999</v>
@@ -13189,7 +13083,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.95</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>80.37</v>
@@ -13249,7 +13143,7 @@
         <v>0.02</v>
       </c>
       <c r="K3" t="n">
-        <v>0.85</v>
+        <v>0.21</v>
       </c>
       <c r="L3" t="n">
         <v>15.14</v>
@@ -13309,7 +13203,7 @@
         <v>0.01</v>
       </c>
       <c r="K4" t="n">
-        <v>2.84</v>
+        <v>0.57</v>
       </c>
       <c r="L4" t="n">
         <v>97.15000000000001</v>
@@ -13369,7 +13263,7 @@
         <v>0.01</v>
       </c>
       <c r="K5" t="n">
-        <v>1.37</v>
+        <v>0.46</v>
       </c>
       <c r="L5" t="n">
         <v>78.81999999999999</v>
@@ -13429,7 +13323,7 @@
         <v>0.01</v>
       </c>
       <c r="K6" t="n">
-        <v>1.96</v>
+        <v>0.49</v>
       </c>
       <c r="L6" t="n">
         <v>84.65000000000001</v>
@@ -13489,7 +13383,7 @@
         <v>0.02</v>
       </c>
       <c r="K7" t="n">
-        <v>2.28</v>
+        <v>1.14</v>
       </c>
       <c r="L7" t="n">
         <v>98.72</v>
@@ -13549,7 +13443,7 @@
         <v>0.02</v>
       </c>
       <c r="K8" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="L8" t="n">
         <v>29.32</v>
@@ -13765,7 +13659,7 @@
         <v>0.04</v>
       </c>
       <c r="K3" t="n">
-        <v>2.21</v>
+        <v>1.47</v>
       </c>
       <c r="L3" t="n">
         <v>53.01</v>
@@ -13825,7 +13719,7 @@
         <v>0.04</v>
       </c>
       <c r="K4" t="n">
-        <v>2.16</v>
+        <v>1.44</v>
       </c>
       <c r="L4" t="n">
         <v>51.87</v>
@@ -13885,7 +13779,7 @@
         <v>0.04</v>
       </c>
       <c r="K5" t="n">
-        <v>4.09</v>
+        <v>2.73</v>
       </c>
       <c r="L5" t="n">
         <v>98.91</v>
@@ -14041,7 +13935,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>66</v>
@@ -14101,7 +13995,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>2.36</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>97.28</v>
@@ -14161,7 +14055,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>4.85</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>160.14</v>
@@ -14221,7 +14115,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>2.18</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>51.28</v>
@@ -14281,7 +14175,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>3.95</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>93.08</v>
@@ -14341,7 +14235,7 @@
         <v>0.01</v>
       </c>
       <c r="K7" t="n">
-        <v>2.37</v>
+        <v>0.47</v>
       </c>
       <c r="L7" t="n">
         <v>80.04000000000001</v>
@@ -14401,7 +14295,7 @@
         <v>0.03</v>
       </c>
       <c r="K8" t="n">
-        <v>2.11</v>
+        <v>0.91</v>
       </c>
       <c r="L8" t="n">
         <v>43.18</v>
@@ -14521,7 +14415,7 @@
         <v>0.03</v>
       </c>
       <c r="K10" t="n">
-        <v>2.04</v>
+        <v>0.87</v>
       </c>
       <c r="L10" t="n">
         <v>41.58</v>
@@ -14581,7 +14475,7 @@
         <v>0.01</v>
       </c>
       <c r="K11" t="n">
-        <v>1.7</v>
+        <v>0.57</v>
       </c>
       <c r="L11" t="n">
         <v>98.09</v>
@@ -14641,7 +14535,7 @@
         <v>0.01</v>
       </c>
       <c r="K12" t="n">
-        <v>3.85</v>
+        <v>1.28</v>
       </c>
       <c r="L12" t="n">
         <v>221.94</v>
@@ -14701,7 +14595,7 @@
         <v>0.01</v>
       </c>
       <c r="K13" t="n">
-        <v>1.41</v>
+        <v>0.47</v>
       </c>
       <c r="L13" t="n">
         <v>81.48999999999999</v>
@@ -14761,7 +14655,7 @@
         <v>0.01</v>
       </c>
       <c r="K14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
         <v>173</v>
@@ -14821,7 +14715,7 @@
         <v>0.01</v>
       </c>
       <c r="K15" t="n">
-        <v>1.02</v>
+        <v>0.34</v>
       </c>
       <c r="L15" t="n">
         <v>58.98</v>
@@ -14881,7 +14775,7 @@
         <v>0.01</v>
       </c>
       <c r="K16" t="n">
-        <v>2.36</v>
+        <v>0.79</v>
       </c>
       <c r="L16" t="n">
         <v>136.08</v>
@@ -14941,7 +14835,7 @@
         <v>0.01</v>
       </c>
       <c r="K17" t="n">
-        <v>2.56</v>
+        <v>0.64</v>
       </c>
       <c r="L17" t="n">
         <v>110.72</v>
@@ -15001,7 +14895,7 @@
         <v>0.03</v>
       </c>
       <c r="K18" t="n">
-        <v>1.46</v>
+        <v>0.63</v>
       </c>
       <c r="L18" t="n">
         <v>29.85</v>
@@ -15061,7 +14955,7 @@
         <v>0.01</v>
       </c>
       <c r="K19" t="n">
-        <v>2.41</v>
+        <v>0.6</v>
       </c>
       <c r="L19" t="n">
         <v>104.07</v>
@@ -15121,7 +15015,7 @@
         <v>0.01</v>
       </c>
       <c r="K20" t="n">
-        <v>2.04</v>
+        <v>0.51</v>
       </c>
       <c r="L20" t="n">
         <v>88.12</v>
@@ -15181,7 +15075,7 @@
         <v>0.02</v>
       </c>
       <c r="K21" t="n">
-        <v>4.7</v>
+        <v>2.35</v>
       </c>
       <c r="L21" t="n">
         <v>203.17</v>
@@ -15241,7 +15135,7 @@
         <v>0.02</v>
       </c>
       <c r="K22" t="n">
-        <v>3.17</v>
+        <v>1.59</v>
       </c>
       <c r="L22" t="n">
         <v>137.17</v>
@@ -15301,7 +15195,7 @@
         <v>0.03</v>
       </c>
       <c r="K23" t="n">
-        <v>0.71</v>
+        <v>0.3</v>
       </c>
       <c r="L23" t="n">
         <v>14.47</v>
@@ -15361,7 +15255,7 @@
         <v>0.02</v>
       </c>
       <c r="K24" t="n">
-        <v>2.44</v>
+        <v>1.22</v>
       </c>
       <c r="L24" t="n">
         <v>105.37</v>
@@ -15421,7 +15315,7 @@
         <v>0.02</v>
       </c>
       <c r="K25" t="n">
-        <v>1.01</v>
+        <v>0.67</v>
       </c>
       <c r="L25" t="n">
         <v>59.06</v>
@@ -15481,7 +15375,7 @@
         <v>0.03</v>
       </c>
       <c r="K26" t="n">
-        <v>2.8</v>
+        <v>1.2</v>
       </c>
       <c r="L26" t="n">
         <v>57.6</v>
@@ -15541,7 +15435,7 @@
         <v>0.02</v>
       </c>
       <c r="K27" t="n">
-        <v>1.86</v>
+        <v>1.24</v>
       </c>
       <c r="L27" t="n">
         <v>109.27</v>
@@ -15601,7 +15495,7 @@
         <v>0.03</v>
       </c>
       <c r="K28" t="n">
-        <v>3.46</v>
+        <v>1.48</v>
       </c>
       <c r="L28" t="n">
         <v>71.12</v>
@@ -15661,7 +15555,7 @@
         <v>0.02</v>
       </c>
       <c r="K29" t="n">
-        <v>2.2</v>
+        <v>1.46</v>
       </c>
       <c r="L29" t="n">
         <v>128.83</v>
@@ -15721,7 +15615,7 @@
         <v>0.02</v>
       </c>
       <c r="K30" t="n">
-        <v>3.07</v>
+        <v>2.04</v>
       </c>
       <c r="L30" t="n">
         <v>179.82</v>
@@ -15781,7 +15675,7 @@
         <v>0.02</v>
       </c>
       <c r="K31" t="n">
-        <v>2.94</v>
+        <v>1.96</v>
       </c>
       <c r="L31" t="n">
         <v>172.19</v>
@@ -15841,7 +15735,7 @@
         <v>0.02</v>
       </c>
       <c r="K32" t="n">
-        <v>1.21</v>
+        <v>0.8</v>
       </c>
       <c r="L32" t="n">
         <v>70.8</v>
@@ -15997,7 +15891,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>4.52</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>106.54</v>
@@ -16153,7 +16047,7 @@
         <v>0.03</v>
       </c>
       <c r="K2" t="n">
-        <v>1.65</v>
+        <v>0.83</v>
       </c>
       <c r="L2" t="n">
         <v>39.44</v>
@@ -16212,9 +16106,7 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>11.94</v>
       </c>
@@ -16273,7 +16165,7 @@
         <v>0.03</v>
       </c>
       <c r="K4" t="n">
-        <v>1.05</v>
+        <v>0.63</v>
       </c>
       <c r="L4" t="n">
         <v>30.03</v>
@@ -16333,7 +16225,7 @@
         <v>0.03</v>
       </c>
       <c r="K5" t="n">
-        <v>1.78</v>
+        <v>1.07</v>
       </c>
       <c r="L5" t="n">
         <v>50.83</v>
@@ -16393,7 +16285,7 @@
         <v>0.03</v>
       </c>
       <c r="K6" t="n">
-        <v>1.91</v>
+        <v>0.72</v>
       </c>
       <c r="L6" t="n">
         <v>34.13</v>
@@ -16453,7 +16345,7 @@
         <v>0.03</v>
       </c>
       <c r="K7" t="n">
-        <v>2.23</v>
+        <v>0.84</v>
       </c>
       <c r="L7" t="n">
         <v>39.9</v>
@@ -16513,7 +16405,7 @@
         <v>0.03</v>
       </c>
       <c r="K8" t="n">
-        <v>2.33</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
         <v>47.67</v>
@@ -16573,7 +16465,7 @@
         <v>0.03</v>
       </c>
       <c r="K9" t="n">
-        <v>2.01</v>
+        <v>0.86</v>
       </c>
       <c r="L9" t="n">
         <v>41.09</v>
@@ -16633,7 +16525,7 @@
         <v>0.03</v>
       </c>
       <c r="K10" t="n">
-        <v>1.06</v>
+        <v>0.4</v>
       </c>
       <c r="L10" t="n">
         <v>18.93</v>
@@ -16693,7 +16585,7 @@
         <v>0.09</v>
       </c>
       <c r="K11" t="n">
-        <v>11.66</v>
+        <v>5.25</v>
       </c>
       <c r="L11" t="n">
         <v>107.83</v>
@@ -16848,9 +16740,7 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>38</v>
       </c>
@@ -16908,9 +16798,7 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>29.92</v>
       </c>
@@ -16968,9 +16856,7 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>40.83</v>
       </c>
@@ -17029,7 +16915,7 @@
         <v>0.01</v>
       </c>
       <c r="K5" t="n">
-        <v>1.25</v>
+        <v>0.42</v>
       </c>
       <c r="L5" t="n">
         <v>72.3</v>
@@ -17088,9 +16974,7 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>28.63</v>
       </c>
@@ -17148,9 +17032,7 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>32.85</v>
       </c>
@@ -17208,9 +17090,7 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>32.64</v>
       </c>
@@ -17269,7 +17149,7 @@
         <v>0.01</v>
       </c>
       <c r="K9" t="n">
-        <v>1.67</v>
+        <v>0.42</v>
       </c>
       <c r="L9" t="n">
         <v>72.31999999999999</v>
@@ -17328,9 +17208,7 @@
       <c r="J10" t="n">
         <v>0</v>
       </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
         <v>34.09</v>
       </c>
@@ -17389,7 +17267,7 @@
         <v>0.02</v>
       </c>
       <c r="K11" t="n">
-        <v>1.03</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L11" t="n">
         <v>60.33</v>
@@ -17449,7 +17327,7 @@
         <v>0.02</v>
       </c>
       <c r="K12" t="n">
-        <v>1.93</v>
+        <v>0.77</v>
       </c>
       <c r="L12" t="n">
         <v>68.03</v>
@@ -17508,9 +17386,7 @@
       <c r="J13" t="n">
         <v>0</v>
       </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
         <v>39.23</v>
       </c>
@@ -17665,7 +17541,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.59</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>65.55</v>
@@ -17725,7 +17601,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>2.22</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>91.45999999999999</v>
@@ -17785,7 +17661,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>4.1</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>135.14</v>
@@ -17845,7 +17721,7 @@
         <v>0.03</v>
       </c>
       <c r="K5" t="n">
-        <v>1.56</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L5" t="n">
         <v>44.75</v>
@@ -17905,7 +17781,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>3.81</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>89.81</v>
@@ -17965,7 +17841,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>4.9</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>115.5</v>
@@ -18025,7 +17901,7 @@
         <v>0.01</v>
       </c>
       <c r="K8" t="n">
-        <v>6.9</v>
+        <v>2.3</v>
       </c>
       <c r="L8" t="n">
         <v>397.9</v>
@@ -18085,7 +17961,7 @@
         <v>0.01</v>
       </c>
       <c r="K9" t="n">
-        <v>6.6</v>
+        <v>2.2</v>
       </c>
       <c r="L9" t="n">
         <v>380.6</v>
@@ -18145,7 +18021,7 @@
         <v>0.01</v>
       </c>
       <c r="K10" t="n">
-        <v>7.2</v>
+        <v>2.4</v>
       </c>
       <c r="L10" t="n">
         <v>415.2</v>
@@ -18205,7 +18081,7 @@
         <v>0.01</v>
       </c>
       <c r="K11" t="n">
-        <v>6.5</v>
+        <v>2.17</v>
       </c>
       <c r="L11" t="n">
         <v>374.96</v>
@@ -18265,7 +18141,7 @@
         <v>0.03</v>
       </c>
       <c r="K12" t="n">
-        <v>2.47</v>
+        <v>1.06</v>
       </c>
       <c r="L12" t="n">
         <v>50.49</v>
@@ -18325,7 +18201,7 @@
         <v>0.01</v>
       </c>
       <c r="K13" t="n">
-        <v>2.87</v>
+        <v>0.96</v>
       </c>
       <c r="L13" t="n">
         <v>165.67</v>
@@ -18385,7 +18261,7 @@
         <v>0.01</v>
       </c>
       <c r="K14" t="n">
-        <v>1.89</v>
+        <v>0.63</v>
       </c>
       <c r="L14" t="n">
         <v>108.87</v>
@@ -18445,7 +18321,7 @@
         <v>0.01</v>
       </c>
       <c r="K15" t="n">
-        <v>6.84</v>
+        <v>2.28</v>
       </c>
       <c r="L15" t="n">
         <v>394.44</v>
@@ -18505,7 +18381,7 @@
         <v>0.01</v>
       </c>
       <c r="K16" t="n">
-        <v>11.31</v>
+        <v>3.77</v>
       </c>
       <c r="L16" t="n">
         <v>652.21</v>
@@ -18565,7 +18441,7 @@
         <v>0.01</v>
       </c>
       <c r="K17" t="n">
-        <v>1.65</v>
+        <v>0.55</v>
       </c>
       <c r="L17" t="n">
         <v>95.15000000000001</v>
@@ -18625,7 +18501,7 @@
         <v>0.03</v>
       </c>
       <c r="K18" t="n">
-        <v>2.88</v>
+        <v>1.23</v>
       </c>
       <c r="L18" t="n">
         <v>58.76</v>
@@ -18685,7 +18561,7 @@
         <v>0.01</v>
       </c>
       <c r="K19" t="n">
-        <v>11.6</v>
+        <v>2.9</v>
       </c>
       <c r="L19" t="n">
         <v>501.7</v>
@@ -18745,7 +18621,7 @@
         <v>0.01</v>
       </c>
       <c r="K20" t="n">
-        <v>9.4</v>
+        <v>2.35</v>
       </c>
       <c r="L20" t="n">
         <v>406.55</v>
@@ -18805,7 +18681,7 @@
         <v>0.01</v>
       </c>
       <c r="K21" t="n">
-        <v>10.12</v>
+        <v>2.53</v>
       </c>
       <c r="L21" t="n">
         <v>437.69</v>
@@ -18865,7 +18741,7 @@
         <v>0.02</v>
       </c>
       <c r="K22" t="n">
-        <v>1.71</v>
+        <v>0.86</v>
       </c>
       <c r="L22" t="n">
         <v>73.98</v>
@@ -18925,7 +18801,7 @@
         <v>0.02</v>
       </c>
       <c r="K23" t="n">
-        <v>8.9</v>
+        <v>4.45</v>
       </c>
       <c r="L23" t="n">
         <v>384.85</v>
@@ -18985,7 +18861,7 @@
         <v>0.02</v>
       </c>
       <c r="K24" t="n">
-        <v>6.4</v>
+        <v>3.2</v>
       </c>
       <c r="L24" t="n">
         <v>276.87</v>
@@ -19045,7 +18921,7 @@
         <v>0.03</v>
       </c>
       <c r="K25" t="n">
-        <v>2.31</v>
+        <v>0.99</v>
       </c>
       <c r="L25" t="n">
         <v>47.1</v>
@@ -19105,7 +18981,7 @@
         <v>0.09</v>
       </c>
       <c r="K26" t="n">
-        <v>10.34</v>
+        <v>5.17</v>
       </c>
       <c r="L26" t="n">
         <v>105.69</v>
@@ -19165,7 +19041,7 @@
         <v>0.02</v>
       </c>
       <c r="K27" t="n">
-        <v>3.25</v>
+        <v>1.08</v>
       </c>
       <c r="L27" t="n">
         <v>93.68000000000001</v>
@@ -19225,7 +19101,7 @@
         <v>0.03</v>
       </c>
       <c r="K28" t="n">
-        <v>5.41</v>
+        <v>1.8</v>
       </c>
       <c r="L28" t="n">
         <v>85.98999999999999</v>
@@ -19285,7 +19161,7 @@
         <v>0.02</v>
       </c>
       <c r="K29" t="n">
-        <v>6.78</v>
+        <v>4.52</v>
       </c>
       <c r="L29" t="n">
         <v>397.76</v>
@@ -19345,7 +19221,7 @@
         <v>0.02</v>
       </c>
       <c r="K30" t="n">
-        <v>6.15</v>
+        <v>4.1</v>
       </c>
       <c r="L30" t="n">
         <v>360.8</v>
@@ -19405,7 +19281,7 @@
         <v>0.02</v>
       </c>
       <c r="K31" t="n">
-        <v>9.42</v>
+        <v>6.28</v>
       </c>
       <c r="L31" t="n">
         <v>552.66</v>
@@ -19465,7 +19341,7 @@
         <v>0.03</v>
       </c>
       <c r="K32" t="n">
-        <v>2.98</v>
+        <v>1.28</v>
       </c>
       <c r="L32" t="n">
         <v>61.3</v>
@@ -19525,7 +19401,7 @@
         <v>0.02</v>
       </c>
       <c r="K33" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L33" t="n">
         <v>352.04</v>
@@ -19585,7 +19461,7 @@
         <v>0.02</v>
       </c>
       <c r="K34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L34" t="n">
         <v>176</v>
@@ -19645,7 +19521,7 @@
         <v>0.02</v>
       </c>
       <c r="K35" t="n">
-        <v>8.57</v>
+        <v>4.29</v>
       </c>
       <c r="L35" t="n">
         <v>377.26</v>
@@ -19705,7 +19581,7 @@
         <v>0.02</v>
       </c>
       <c r="K36" t="n">
-        <v>7.68</v>
+        <v>3.84</v>
       </c>
       <c r="L36" t="n">
         <v>337.92</v>
@@ -19765,7 +19641,7 @@
         <v>0.02</v>
       </c>
       <c r="K37" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L37" t="n">
         <v>352</v>
@@ -19825,7 +19701,7 @@
         <v>0.02</v>
       </c>
       <c r="K38" t="n">
-        <v>8.16</v>
+        <v>4.08</v>
       </c>
       <c r="L38" t="n">
         <v>359.15</v>
@@ -19981,7 +19857,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>4.3</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>101.36</v>
@@ -20137,7 +20013,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.86</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>76.53</v>
@@ -20197,7 +20073,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>2.36</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>97.53</v>
@@ -20257,7 +20133,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>94.34</v>
@@ -20317,7 +20193,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>89.05</v>
@@ -20377,7 +20253,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>3.53</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>116.64</v>
@@ -20437,7 +20313,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>2.92</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>96.31</v>
@@ -20497,7 +20373,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
         <v>75.52</v>
@@ -20557,7 +20433,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>3.62</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
         <v>119.4</v>
@@ -20617,7 +20493,7 @@
         <v>0.03</v>
       </c>
       <c r="K10" t="n">
-        <v>1.89</v>
+        <v>0.95</v>
       </c>
       <c r="L10" t="n">
         <v>45.12</v>
@@ -20677,7 +20553,7 @@
         <v>0.01</v>
       </c>
       <c r="K11" t="n">
-        <v>1.84</v>
+        <v>0.61</v>
       </c>
       <c r="L11" t="n">
         <v>105.82</v>
@@ -20737,7 +20613,7 @@
         <v>0.01</v>
       </c>
       <c r="K12" t="n">
-        <v>1.4</v>
+        <v>0.46</v>
       </c>
       <c r="L12" t="n">
         <v>80.44</v>
@@ -20797,7 +20673,7 @@
         <v>0.01</v>
       </c>
       <c r="K13" t="n">
-        <v>7.69</v>
+        <v>2.56</v>
       </c>
       <c r="L13" t="n">
         <v>443.27</v>
@@ -20857,7 +20733,7 @@
         <v>0.01</v>
       </c>
       <c r="K14" t="n">
-        <v>1.88</v>
+        <v>0.63</v>
       </c>
       <c r="L14" t="n">
         <v>108.46</v>
@@ -20917,7 +20793,7 @@
         <v>0.01</v>
       </c>
       <c r="K15" t="n">
-        <v>1.89</v>
+        <v>0.63</v>
       </c>
       <c r="L15" t="n">
         <v>109.08</v>
@@ -20977,7 +20853,7 @@
         <v>0.01</v>
       </c>
       <c r="K16" t="n">
-        <v>2.12</v>
+        <v>0.71</v>
       </c>
       <c r="L16" t="n">
         <v>122.53</v>
@@ -21037,7 +20913,7 @@
         <v>0.03</v>
       </c>
       <c r="K17" t="n">
-        <v>2.59</v>
+        <v>1.11</v>
       </c>
       <c r="L17" t="n">
         <v>52.94</v>
@@ -21096,9 +20972,7 @@
       <c r="J18" t="n">
         <v>0</v>
       </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
         <v>17.84</v>
       </c>
@@ -21157,7 +21031,7 @@
         <v>0.01</v>
       </c>
       <c r="K19" t="n">
-        <v>0.57</v>
+        <v>0.19</v>
       </c>
       <c r="L19" t="n">
         <v>32.76</v>
@@ -21217,7 +21091,7 @@
         <v>0.01</v>
       </c>
       <c r="K20" t="n">
-        <v>2.13</v>
+        <v>0.71</v>
       </c>
       <c r="L20" t="n">
         <v>122.67</v>
@@ -21277,7 +21151,7 @@
         <v>0.01</v>
       </c>
       <c r="K21" t="n">
-        <v>1.7</v>
+        <v>0.42</v>
       </c>
       <c r="L21" t="n">
         <v>73.33</v>
@@ -21337,7 +21211,7 @@
         <v>0.01</v>
       </c>
       <c r="K22" t="n">
-        <v>2.1</v>
+        <v>0.53</v>
       </c>
       <c r="L22" t="n">
         <v>90.98</v>
@@ -21397,7 +21271,7 @@
         <v>0.01</v>
       </c>
       <c r="K23" t="n">
-        <v>3.18</v>
+        <v>0.8</v>
       </c>
       <c r="L23" t="n">
         <v>137.59</v>
@@ -21457,7 +21331,7 @@
         <v>0.03</v>
       </c>
       <c r="K24" t="n">
-        <v>2.03</v>
+        <v>0.87</v>
       </c>
       <c r="L24" t="n">
         <v>41.37</v>
@@ -21517,7 +21391,7 @@
         <v>0.01</v>
       </c>
       <c r="K25" t="n">
-        <v>2.41</v>
+        <v>0.6</v>
       </c>
       <c r="L25" t="n">
         <v>104.06</v>
@@ -21577,7 +21451,7 @@
         <v>0.01</v>
       </c>
       <c r="K26" t="n">
-        <v>2.39</v>
+        <v>0.6</v>
       </c>
       <c r="L26" t="n">
         <v>103.42</v>
@@ -21637,7 +21511,7 @@
         <v>0.01</v>
       </c>
       <c r="K27" t="n">
-        <v>2.58</v>
+        <v>0.64</v>
       </c>
       <c r="L27" t="n">
         <v>111.43</v>
@@ -21697,7 +21571,7 @@
         <v>0.02</v>
       </c>
       <c r="K28" t="n">
-        <v>0.61</v>
+        <v>0.31</v>
       </c>
       <c r="L28" t="n">
         <v>26.52</v>
@@ -21757,7 +21631,7 @@
         <v>0.02</v>
       </c>
       <c r="K29" t="n">
-        <v>1.81</v>
+        <v>0.9</v>
       </c>
       <c r="L29" t="n">
         <v>78.14</v>
@@ -21817,7 +21691,7 @@
         <v>0.02</v>
       </c>
       <c r="K30" t="n">
-        <v>2.1</v>
+        <v>1.05</v>
       </c>
       <c r="L30" t="n">
         <v>90.95</v>
@@ -21877,7 +21751,7 @@
         <v>0.02</v>
       </c>
       <c r="K31" t="n">
-        <v>3.07</v>
+        <v>1.54</v>
       </c>
       <c r="L31" t="n">
         <v>132.87</v>
@@ -21937,7 +21811,7 @@
         <v>0.02</v>
       </c>
       <c r="K32" t="n">
-        <v>2.34</v>
+        <v>1.17</v>
       </c>
       <c r="L32" t="n">
         <v>101.31</v>
@@ -21997,7 +21871,7 @@
         <v>0.02</v>
       </c>
       <c r="K33" t="n">
-        <v>3.03</v>
+        <v>1.51</v>
       </c>
       <c r="L33" t="n">
         <v>131.01</v>
@@ -22057,7 +21931,7 @@
         <v>0.02</v>
       </c>
       <c r="K34" t="n">
-        <v>2.63</v>
+        <v>1.31</v>
       </c>
       <c r="L34" t="n">
         <v>113.55</v>
@@ -22117,7 +21991,7 @@
         <v>0.02</v>
       </c>
       <c r="K35" t="n">
-        <v>2.2</v>
+        <v>1.47</v>
       </c>
       <c r="L35" t="n">
         <v>126.76</v>
@@ -22177,7 +22051,7 @@
         <v>0.02</v>
       </c>
       <c r="K36" t="n">
-        <v>2.29</v>
+        <v>1.15</v>
       </c>
       <c r="L36" t="n">
         <v>99.22</v>
@@ -22237,7 +22111,7 @@
         <v>0.02</v>
       </c>
       <c r="K37" t="n">
-        <v>2.58</v>
+        <v>1.29</v>
       </c>
       <c r="L37" t="n">
         <v>111.66</v>
@@ -22297,7 +22171,7 @@
         <v>0.02</v>
       </c>
       <c r="K38" t="n">
-        <v>3.05</v>
+        <v>1.02</v>
       </c>
       <c r="L38" t="n">
         <v>87.84999999999999</v>
@@ -22357,7 +22231,7 @@
         <v>0.02</v>
       </c>
       <c r="K39" t="n">
-        <v>1.53</v>
+        <v>1.02</v>
       </c>
       <c r="L39" t="n">
         <v>89.83</v>
@@ -22417,7 +22291,7 @@
         <v>0.02</v>
       </c>
       <c r="K40" t="n">
-        <v>1.53</v>
+        <v>1.02</v>
       </c>
       <c r="L40" t="n">
         <v>89.70999999999999</v>
@@ -22477,7 +22351,7 @@
         <v>0.02</v>
       </c>
       <c r="K41" t="n">
-        <v>2.01</v>
+        <v>1.34</v>
       </c>
       <c r="L41" t="n">
         <v>118.03</v>
@@ -22537,7 +22411,7 @@
         <v>0.02</v>
       </c>
       <c r="K42" t="n">
-        <v>1.05</v>
+        <v>0.53</v>
       </c>
       <c r="L42" t="n">
         <v>46.41</v>
@@ -22597,7 +22471,7 @@
         <v>0.02</v>
       </c>
       <c r="K43" t="n">
-        <v>2.08</v>
+        <v>1.04</v>
       </c>
       <c r="L43" t="n">
         <v>91.52</v>
@@ -22657,7 +22531,7 @@
         <v>0.02</v>
       </c>
       <c r="K44" t="n">
-        <v>1.95</v>
+        <v>0.97</v>
       </c>
       <c r="L44" t="n">
         <v>85.59999999999999</v>
@@ -22717,7 +22591,7 @@
         <v>0.02</v>
       </c>
       <c r="K45" t="n">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="L45" t="n">
         <v>79.25</v>
@@ -22777,7 +22651,7 @@
         <v>0.02</v>
       </c>
       <c r="K46" t="n">
-        <v>2.5</v>
+        <v>1.25</v>
       </c>
       <c r="L46" t="n">
         <v>110.04</v>
@@ -22837,7 +22711,7 @@
         <v>0.02</v>
       </c>
       <c r="K47" t="n">
-        <v>2.39</v>
+        <v>1.19</v>
       </c>
       <c r="L47" t="n">
         <v>104.96</v>
@@ -22897,7 +22771,7 @@
         <v>0.02</v>
       </c>
       <c r="K48" t="n">
-        <v>2.02</v>
+        <v>1.01</v>
       </c>
       <c r="L48" t="n">
         <v>88.83</v>
@@ -22957,7 +22831,7 @@
         <v>0.02</v>
       </c>
       <c r="K49" t="n">
-        <v>1.37</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L49" t="n">
         <v>60.3</v>
@@ -23017,7 +22891,7 @@
         <v>0.02</v>
       </c>
       <c r="K50" t="n">
-        <v>2.05</v>
+        <v>1.03</v>
       </c>
       <c r="L50" t="n">
         <v>90.31</v>
@@ -23077,7 +22951,7 @@
         <v>0.03</v>
       </c>
       <c r="K51" t="n">
-        <v>0.55</v>
+        <v>0.24</v>
       </c>
       <c r="L51" t="n">
         <v>11.32</v>
@@ -23136,9 +23010,7 @@
       <c r="J52" t="n">
         <v>0</v>
       </c>
-      <c r="K52" t="n">
-        <v>0</v>
-      </c>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" t="n">
         <v>19.49</v>
       </c>
@@ -23197,7 +23069,7 @@
         <v>0.03</v>
       </c>
       <c r="K53" t="n">
-        <v>2.03</v>
+        <v>0.87</v>
       </c>
       <c r="L53" t="n">
         <v>41.78</v>
@@ -23257,7 +23129,7 @@
         <v>0.02</v>
       </c>
       <c r="K54" t="n">
-        <v>1.71</v>
+        <v>0.86</v>
       </c>
       <c r="L54" t="n">
         <v>75.31</v>
@@ -23317,7 +23189,7 @@
         <v>0.03</v>
       </c>
       <c r="K55" t="n">
-        <v>2.21</v>
+        <v>0.83</v>
       </c>
       <c r="L55" t="n">
         <v>39.79</v>
@@ -23473,7 +23345,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>2.81</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>92.59</v>
@@ -23533,7 +23405,7 @@
         <v>0.01</v>
       </c>
       <c r="K3" t="n">
-        <v>3.44</v>
+        <v>0.49</v>
       </c>
       <c r="L3" t="n">
         <v>82.94</v>
@@ -23593,7 +23465,7 @@
         <v>0.02</v>
       </c>
       <c r="K4" t="n">
-        <v>1.78</v>
+        <v>0.89</v>
       </c>
       <c r="L4" t="n">
         <v>77.13</v>
@@ -23653,7 +23525,7 @@
         <v>0.02</v>
       </c>
       <c r="K5" t="n">
-        <v>2.49</v>
+        <v>1.25</v>
       </c>
       <c r="L5" t="n">
         <v>107.83</v>
@@ -23713,7 +23585,7 @@
         <v>0.02</v>
       </c>
       <c r="K6" t="n">
-        <v>1.76</v>
+        <v>0.88</v>
       </c>
       <c r="L6" t="n">
         <v>77.56999999999999</v>
@@ -23869,7 +23741,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>2.07</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>85.37</v>
@@ -23929,7 +23801,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1.74</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>71.61</v>
@@ -23989,7 +23861,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1.53</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>63.32</v>
@@ -24049,7 +23921,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>1.09</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>45.05</v>
@@ -24109,7 +23981,7 @@
         <v>0.09</v>
       </c>
       <c r="K6" t="n">
-        <v>10</v>
+        <v>4.5</v>
       </c>
       <c r="L6" t="n">
         <v>87</v>
@@ -24169,7 +24041,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>3.15</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>104</v>
@@ -24229,7 +24101,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>1.93</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
         <v>63.69</v>
@@ -24289,7 +24161,7 @@
         <v>0.09</v>
       </c>
       <c r="K9" t="n">
-        <v>2.34</v>
+        <v>7.01</v>
       </c>
       <c r="L9" t="n">
         <v>132.39</v>
@@ -24349,7 +24221,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>2.08</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
         <v>68.73</v>
@@ -24409,7 +24281,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>3.08</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>101.62</v>
@@ -24469,7 +24341,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>3.89</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
         <v>106.86</v>
@@ -24529,7 +24401,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>3.12</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>73.56999999999999</v>
@@ -24589,7 +24461,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>3.06</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
         <v>72.06999999999999</v>
@@ -24649,7 +24521,7 @@
         <v>0.09</v>
       </c>
       <c r="K15" t="n">
-        <v>2.75</v>
+        <v>8.25</v>
       </c>
       <c r="L15" t="n">
         <v>155.86</v>
@@ -24709,7 +24581,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>2.09</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>49.3</v>
@@ -24769,7 +24641,7 @@
         <v>0.09</v>
       </c>
       <c r="K17" t="n">
-        <v>12.45</v>
+        <v>5.6</v>
       </c>
       <c r="L17" t="n">
         <v>112.7</v>
@@ -24829,7 +24701,7 @@
         <v>0.09</v>
       </c>
       <c r="K18" t="n">
-        <v>11.04</v>
+        <v>4.97</v>
       </c>
       <c r="L18" t="n">
         <v>99.93000000000001</v>
@@ -24889,7 +24761,7 @@
         <v>0.01</v>
       </c>
       <c r="K19" t="n">
-        <v>1.92</v>
+        <v>0.64</v>
       </c>
       <c r="L19" t="n">
         <v>110.95</v>
@@ -24949,7 +24821,7 @@
         <v>0.01</v>
       </c>
       <c r="K20" t="n">
-        <v>0.72</v>
+        <v>0.24</v>
       </c>
       <c r="L20" t="n">
         <v>41.66</v>
@@ -25009,7 +24881,7 @@
         <v>0.09</v>
       </c>
       <c r="K21" t="n">
-        <v>14.44</v>
+        <v>6.5</v>
       </c>
       <c r="L21" t="n">
         <v>130.72</v>
@@ -25069,7 +24941,7 @@
         <v>0.03</v>
       </c>
       <c r="K22" t="n">
-        <v>2.81</v>
+        <v>1.2</v>
       </c>
       <c r="L22" t="n">
         <v>57.42</v>
@@ -25129,7 +25001,7 @@
         <v>0.09</v>
       </c>
       <c r="K23" t="n">
-        <v>8.49</v>
+        <v>3.82</v>
       </c>
       <c r="L23" t="n">
         <v>76.87</v>
@@ -25189,7 +25061,7 @@
         <v>0.01</v>
       </c>
       <c r="K24" t="n">
-        <v>1.35</v>
+        <v>0.45</v>
       </c>
       <c r="L24" t="n">
         <v>77.62</v>
@@ -25249,7 +25121,7 @@
         <v>0.01</v>
       </c>
       <c r="K25" t="n">
-        <v>1.52</v>
+        <v>0.38</v>
       </c>
       <c r="L25" t="n">
         <v>65.65000000000001</v>
@@ -25309,7 +25181,7 @@
         <v>0.01</v>
       </c>
       <c r="K26" t="n">
-        <v>1.42</v>
+        <v>0.36</v>
       </c>
       <c r="L26" t="n">
         <v>61.52</v>
@@ -25369,7 +25241,7 @@
         <v>0.09</v>
       </c>
       <c r="K27" t="n">
-        <v>5.2</v>
+        <v>2.23</v>
       </c>
       <c r="L27" t="n">
         <v>44.8</v>
@@ -25429,7 +25301,7 @@
         <v>0.09</v>
       </c>
       <c r="K28" t="n">
-        <v>5.2</v>
+        <v>2.23</v>
       </c>
       <c r="L28" t="n">
         <v>44.84</v>
@@ -25489,7 +25361,7 @@
         <v>0.09</v>
       </c>
       <c r="K29" t="n">
-        <v>7.35</v>
+        <v>3.15</v>
       </c>
       <c r="L29" t="n">
         <v>63.35</v>
@@ -25549,7 +25421,7 @@
         <v>0.02</v>
       </c>
       <c r="K30" t="n">
-        <v>2.09</v>
+        <v>1.05</v>
       </c>
       <c r="L30" t="n">
         <v>90.56999999999999</v>
@@ -25609,7 +25481,7 @@
         <v>0.02</v>
       </c>
       <c r="K31" t="n">
-        <v>1.74</v>
+        <v>0.87</v>
       </c>
       <c r="L31" t="n">
         <v>75.43000000000001</v>
@@ -25669,7 +25541,7 @@
         <v>0.02</v>
       </c>
       <c r="K32" t="n">
-        <v>1.23</v>
+        <v>0.61</v>
       </c>
       <c r="L32" t="n">
         <v>53.18</v>
@@ -25729,7 +25601,7 @@
         <v>0.09</v>
       </c>
       <c r="K33" t="n">
-        <v>8.76</v>
+        <v>4.38</v>
       </c>
       <c r="L33" t="n">
         <v>89.53</v>
@@ -25789,7 +25661,7 @@
         <v>0.02</v>
       </c>
       <c r="K34" t="n">
-        <v>2.32</v>
+        <v>1.16</v>
       </c>
       <c r="L34" t="n">
         <v>100.53</v>
@@ -25849,7 +25721,7 @@
         <v>0.02</v>
       </c>
       <c r="K35" t="n">
-        <v>3.6</v>
+        <v>1.8</v>
       </c>
       <c r="L35" t="n">
         <v>155.77</v>
@@ -25909,7 +25781,7 @@
         <v>0.02</v>
       </c>
       <c r="K36" t="n">
-        <v>1.13</v>
+        <v>0.57</v>
       </c>
       <c r="L36" t="n">
         <v>49.07</v>
@@ -25969,7 +25841,7 @@
         <v>0.02</v>
       </c>
       <c r="K37" t="n">
-        <v>3.75</v>
+        <v>1.25</v>
       </c>
       <c r="L37" t="n">
         <v>108.05</v>
@@ -26029,7 +25901,7 @@
         <v>0.09</v>
       </c>
       <c r="K38" t="n">
-        <v>13.02</v>
+        <v>5.86</v>
       </c>
       <c r="L38" t="n">
         <v>119.76</v>
@@ -26089,7 +25961,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K39" t="n">
-        <v>4.69</v>
+        <v>6.57</v>
       </c>
       <c r="L39" t="n">
         <v>160.56</v>
@@ -26149,7 +26021,7 @@
         <v>0.02</v>
       </c>
       <c r="K40" t="n">
-        <v>1.05</v>
+        <v>0.7</v>
       </c>
       <c r="L40" t="n">
         <v>61.64</v>
@@ -26209,7 +26081,7 @@
         <v>0.02</v>
       </c>
       <c r="K41" t="n">
-        <v>1.06</v>
+        <v>0.71</v>
       </c>
       <c r="L41" t="n">
         <v>62.31</v>
@@ -26268,9 +26140,7 @@
       <c r="J42" t="n">
         <v>0</v>
       </c>
-      <c r="K42" t="n">
-        <v>0</v>
-      </c>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" t="n">
         <v>25.96</v>
       </c>
@@ -26329,7 +26199,7 @@
         <v>0.02</v>
       </c>
       <c r="K43" t="n">
-        <v>1.74</v>
+        <v>1.16</v>
       </c>
       <c r="L43" t="n">
         <v>102.35</v>
@@ -26389,7 +26259,7 @@
         <v>0.02</v>
       </c>
       <c r="K44" t="n">
-        <v>1.42</v>
+        <v>0.95</v>
       </c>
       <c r="L44" t="n">
         <v>83.39</v>
@@ -26449,7 +26319,7 @@
         <v>0.09</v>
       </c>
       <c r="K45" t="n">
-        <v>12.85</v>
+        <v>6.09</v>
       </c>
       <c r="L45" t="n">
         <v>125.09</v>
@@ -26509,7 +26379,7 @@
         <v>0.02</v>
       </c>
       <c r="K46" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.54</v>
       </c>
       <c r="L46" t="n">
         <v>47.47</v>
@@ -26569,7 +26439,7 @@
         <v>0.02</v>
       </c>
       <c r="K47" t="n">
-        <v>0.97</v>
+        <v>0.65</v>
       </c>
       <c r="L47" t="n">
         <v>57.12</v>
@@ -26629,7 +26499,7 @@
         <v>0.02</v>
       </c>
       <c r="K48" t="n">
-        <v>2.49</v>
+        <v>1.24</v>
       </c>
       <c r="L48" t="n">
         <v>109.42</v>
@@ -26689,7 +26559,7 @@
         <v>0.02</v>
       </c>
       <c r="K49" t="n">
-        <v>1.43</v>
+        <v>0.57</v>
       </c>
       <c r="L49" t="n">
         <v>50.44</v>
@@ -26749,7 +26619,7 @@
         <v>0.02</v>
       </c>
       <c r="K50" t="n">
-        <v>2.3</v>
+        <v>1.15</v>
       </c>
       <c r="L50" t="n">
         <v>100.99</v>
@@ -26905,7 +26775,7 @@
         <v>0.03</v>
       </c>
       <c r="K2" t="n">
-        <v>1.87</v>
+        <v>0.8</v>
       </c>
       <c r="L2" t="n">
         <v>38.12</v>
@@ -27061,7 +26931,7 @@
         <v>0.03</v>
       </c>
       <c r="K2" t="n">
-        <v>2.08</v>
+        <v>1.25</v>
       </c>
       <c r="L2" t="n">
         <v>59.59</v>
@@ -27121,7 +26991,7 @@
         <v>0.03</v>
       </c>
       <c r="K3" t="n">
-        <v>2.85</v>
+        <v>1.22</v>
       </c>
       <c r="L3" t="n">
         <v>58.2</v>
@@ -27277,7 +27147,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>21.75</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>897.36</v>
@@ -27337,7 +27207,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>14.26</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>588.15</v>
@@ -27397,7 +27267,7 @@
         <v>0.01</v>
       </c>
       <c r="K4" t="n">
-        <v>1.55</v>
+        <v>0.31</v>
       </c>
       <c r="L4" t="n">
         <v>52.94</v>
@@ -27457,7 +27327,7 @@
         <v>0.01</v>
       </c>
       <c r="K5" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="L5" t="n">
         <v>1557</v>
@@ -27517,7 +27387,7 @@
         <v>0.01</v>
       </c>
       <c r="K6" t="n">
-        <v>29.7</v>
+        <v>9.9</v>
       </c>
       <c r="L6" t="n">
         <v>1712.7</v>
@@ -27577,7 +27447,7 @@
         <v>0.03</v>
       </c>
       <c r="K7" t="n">
-        <v>3.63</v>
+        <v>1.56</v>
       </c>
       <c r="L7" t="n">
         <v>74.22</v>
@@ -27637,7 +27507,7 @@
         <v>0.02</v>
       </c>
       <c r="K8" t="n">
-        <v>2.22</v>
+        <v>0.74</v>
       </c>
       <c r="L8" t="n">
         <v>64.01000000000001</v>
@@ -27697,7 +27567,7 @@
         <v>0.02</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.67</v>
+        <v>1.34</v>
       </c>
       <c r="L9" t="n">
         <v>117.94</v>
@@ -27757,7 +27627,7 @@
         <v>0.02</v>
       </c>
       <c r="K10" t="n">
-        <v>26.28</v>
+        <v>13.14</v>
       </c>
       <c r="L10" t="n">
         <v>1156.3</v>
@@ -27817,7 +27687,7 @@
         <v>0.02</v>
       </c>
       <c r="K11" t="n">
-        <v>1.65</v>
+        <v>0.66</v>
       </c>
       <c r="L11" t="n">
         <v>58.08</v>
@@ -27973,7 +27843,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0.47</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>19.52</v>
@@ -28033,7 +27903,7 @@
         <v>0.01</v>
       </c>
       <c r="K3" t="n">
-        <v>0.85</v>
+        <v>0.17</v>
       </c>
       <c r="L3" t="n">
         <v>29.21</v>
@@ -28093,7 +27963,7 @@
         <v>0.02</v>
       </c>
       <c r="K4" t="n">
-        <v>0.34</v>
+        <v>0.22</v>
       </c>
       <c r="L4" t="n">
         <v>19.68</v>
@@ -28153,7 +28023,7 @@
         <v>0.02</v>
       </c>
       <c r="K5" t="n">
-        <v>0.36</v>
+        <v>0.18</v>
       </c>
       <c r="L5" t="n">
         <v>15.63</v>
@@ -28213,7 +28083,7 @@
         <v>0.02</v>
       </c>
       <c r="K6" t="n">
-        <v>0.74</v>
+        <v>0.19</v>
       </c>
       <c r="L6" t="n">
         <v>13.29</v>
@@ -28369,7 +28239,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>19.86</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>468.12</v>
@@ -28429,7 +28299,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>4.51</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>106.24</v>
@@ -28489,7 +28359,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>2.35</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>55.49</v>
@@ -28549,7 +28419,7 @@
         <v>0.01</v>
       </c>
       <c r="K5" t="n">
-        <v>1.76</v>
+        <v>0.59</v>
       </c>
       <c r="L5" t="n">
         <v>101.25</v>
@@ -28609,7 +28479,7 @@
         <v>0.01</v>
       </c>
       <c r="K6" t="n">
-        <v>0.93</v>
+        <v>0.31</v>
       </c>
       <c r="L6" t="n">
         <v>53.89</v>
@@ -28669,7 +28539,7 @@
         <v>0.01</v>
       </c>
       <c r="K7" t="n">
-        <v>1.3</v>
+        <v>0.43</v>
       </c>
       <c r="L7" t="n">
         <v>75.03</v>
@@ -28729,7 +28599,7 @@
         <v>0.01</v>
       </c>
       <c r="K8" t="n">
-        <v>1.99</v>
+        <v>0.5</v>
       </c>
       <c r="L8" t="n">
         <v>86.14</v>
@@ -28789,7 +28659,7 @@
         <v>0.01</v>
       </c>
       <c r="K9" t="n">
-        <v>5.66</v>
+        <v>1.42</v>
       </c>
       <c r="L9" t="n">
         <v>244.95</v>
@@ -28849,7 +28719,7 @@
         <v>0.01</v>
       </c>
       <c r="K10" t="n">
-        <v>2.59</v>
+        <v>0.65</v>
       </c>
       <c r="L10" t="n">
         <v>112.07</v>
@@ -28909,7 +28779,7 @@
         <v>0.01</v>
       </c>
       <c r="K11" t="n">
-        <v>1.9</v>
+        <v>0.48</v>
       </c>
       <c r="L11" t="n">
         <v>82.18000000000001</v>
@@ -28969,7 +28839,7 @@
         <v>0.09</v>
       </c>
       <c r="K12" t="n">
-        <v>6.38</v>
+        <v>3.19</v>
       </c>
       <c r="L12" t="n">
         <v>65.19</v>
@@ -29029,7 +28899,7 @@
         <v>0.02</v>
       </c>
       <c r="K13" t="n">
-        <v>1.97</v>
+        <v>0.98</v>
       </c>
       <c r="L13" t="n">
         <v>85.11</v>
@@ -29088,9 +28958,7 @@
       <c r="J14" t="n">
         <v>0</v>
       </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>9.49</v>
       </c>
@@ -29149,7 +29017,7 @@
         <v>0.02</v>
       </c>
       <c r="K15" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="L15" t="n">
         <v>60.62</v>
@@ -29209,7 +29077,7 @@
         <v>0.02</v>
       </c>
       <c r="K16" t="n">
-        <v>1.85</v>
+        <v>0.93</v>
       </c>
       <c r="L16" t="n">
         <v>80.19</v>
@@ -29269,7 +29137,7 @@
         <v>0.02</v>
       </c>
       <c r="K17" t="n">
-        <v>3.97</v>
+        <v>1.98</v>
       </c>
       <c r="L17" t="n">
         <v>171.51</v>
@@ -29329,7 +29197,7 @@
         <v>0.02</v>
       </c>
       <c r="K18" t="n">
-        <v>2.25</v>
+        <v>1.5</v>
       </c>
       <c r="L18" t="n">
         <v>132.27</v>
@@ -29389,7 +29257,7 @@
         <v>0.02</v>
       </c>
       <c r="K19" t="n">
-        <v>10.25</v>
+        <v>6.83</v>
       </c>
       <c r="L19" t="n">
         <v>601.11</v>
@@ -29449,7 +29317,7 @@
         <v>0.02</v>
       </c>
       <c r="K20" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="L20" t="n">
         <v>105.6</v>
@@ -29509,7 +29377,7 @@
         <v>0.02</v>
       </c>
       <c r="K21" t="n">
-        <v>3.33</v>
+        <v>1.67</v>
       </c>
       <c r="L21" t="n">
         <v>146.54</v>
@@ -29569,7 +29437,7 @@
         <v>0.02</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L22" t="n">
         <v>44.07</v>
@@ -29725,7 +29593,7 @@
         <v>0.09</v>
       </c>
       <c r="K2" t="n">
-        <v>5.92</v>
+        <v>2.67</v>
       </c>
       <c r="L2" t="n">
         <v>51.54</v>
@@ -29785,7 +29653,7 @@
         <v>0.09</v>
       </c>
       <c r="K3" t="n">
-        <v>2.06</v>
+        <v>4.63</v>
       </c>
       <c r="L3" t="n">
         <v>87.38</v>
@@ -29845,7 +29713,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>90.75</v>
@@ -29905,7 +29773,7 @@
         <v>0.09</v>
       </c>
       <c r="K5" t="n">
-        <v>0.9399999999999999</v>
+        <v>2.11</v>
       </c>
       <c r="L5" t="n">
         <v>39.83</v>
@@ -29965,7 +29833,7 @@
         <v>0.09</v>
       </c>
       <c r="K6" t="n">
-        <v>1.54</v>
+        <v>4.62</v>
       </c>
       <c r="L6" t="n">
         <v>87.20999999999999</v>
@@ -30024,9 +29892,7 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>6.64</v>
       </c>
@@ -30084,9 +29950,7 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>2.14</v>
       </c>
@@ -30145,7 +30009,7 @@
         <v>0.03</v>
       </c>
       <c r="K9" t="n">
-        <v>0.71</v>
+        <v>0.35</v>
       </c>
       <c r="L9" t="n">
         <v>16.84</v>
@@ -30205,7 +30069,7 @@
         <v>0.03</v>
       </c>
       <c r="K10" t="n">
-        <v>0.88</v>
+        <v>0.53</v>
       </c>
       <c r="L10" t="n">
         <v>25.23</v>
@@ -30265,7 +30129,7 @@
         <v>0.03</v>
       </c>
       <c r="K11" t="n">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="L11" t="n">
         <v>42.83</v>
@@ -30325,7 +30189,7 @@
         <v>0.09</v>
       </c>
       <c r="K12" t="n">
-        <v>0.72</v>
+        <v>1.63</v>
       </c>
       <c r="L12" t="n">
         <v>30.76</v>
@@ -30385,7 +30249,7 @@
         <v>0.09</v>
       </c>
       <c r="K13" t="n">
-        <v>0.93</v>
+        <v>2.79</v>
       </c>
       <c r="L13" t="n">
         <v>52.77</v>
@@ -30445,7 +30309,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>2.35</v>
+        <v>2.74</v>
       </c>
       <c r="L14" t="n">
         <v>66.47</v>
@@ -30505,7 +30369,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>0.58</v>
+        <v>0.67</v>
       </c>
       <c r="L15" t="n">
         <v>16.39</v>
@@ -30565,7 +30429,7 @@
         <v>0.09</v>
       </c>
       <c r="K16" t="n">
-        <v>8.949999999999999</v>
+        <v>4.03</v>
       </c>
       <c r="L16" t="n">
         <v>81.04000000000001</v>
@@ -30625,7 +30489,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>1.47</v>
+        <v>1.71</v>
       </c>
       <c r="L17" t="n">
         <v>41.52</v>
@@ -30685,7 +30549,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>2.59</v>
+        <v>3.63</v>
       </c>
       <c r="L18" t="n">
         <v>88.17</v>
@@ -30745,7 +30609,7 @@
         <v>0.03</v>
       </c>
       <c r="K19" t="n">
-        <v>2.71</v>
+        <v>1.02</v>
       </c>
       <c r="L19" t="n">
         <v>48.48</v>
@@ -30805,7 +30669,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K20" t="n">
-        <v>1.81</v>
+        <v>2.11</v>
       </c>
       <c r="L20" t="n">
         <v>51.32</v>
@@ -30865,7 +30729,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K21" t="n">
-        <v>1.33</v>
+        <v>1.55</v>
       </c>
       <c r="L21" t="n">
         <v>37.64</v>
@@ -30925,7 +30789,7 @@
         <v>0.03</v>
       </c>
       <c r="K22" t="n">
-        <v>2.1</v>
+        <v>0.9</v>
       </c>
       <c r="L22" t="n">
         <v>42.9</v>
@@ -30985,7 +30849,7 @@
         <v>0.03</v>
       </c>
       <c r="K23" t="n">
-        <v>2.47</v>
+        <v>0.93</v>
       </c>
       <c r="L23" t="n">
         <v>44.19</v>
@@ -31045,7 +30909,7 @@
         <v>0.03</v>
       </c>
       <c r="K24" t="n">
-        <v>1.37</v>
+        <v>0.51</v>
       </c>
       <c r="L24" t="n">
         <v>24.53</v>
@@ -31104,9 +30968,7 @@
       <c r="J25" t="n">
         <v>0</v>
       </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
         <v>9.49</v>
       </c>
@@ -31165,7 +31027,7 @@
         <v>0.09</v>
       </c>
       <c r="K26" t="n">
-        <v>4.9</v>
+        <v>2.45</v>
       </c>
       <c r="L26" t="n">
         <v>50.1</v>
@@ -31225,7 +31087,7 @@
         <v>0.09</v>
       </c>
       <c r="K27" t="n">
-        <v>8.73</v>
+        <v>4.37</v>
       </c>
       <c r="L27" t="n">
         <v>89.26000000000001</v>
@@ -31285,7 +31147,7 @@
         <v>0.09</v>
       </c>
       <c r="K28" t="n">
-        <v>3.32</v>
+        <v>1.66</v>
       </c>
       <c r="L28" t="n">
         <v>33.95</v>
@@ -31345,7 +31207,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K29" t="n">
-        <v>1.63</v>
+        <v>1.9</v>
       </c>
       <c r="L29" t="n">
         <v>46.19</v>
@@ -31405,7 +31267,7 @@
         <v>0.09</v>
       </c>
       <c r="K30" t="n">
-        <v>6</v>
+        <v>2.57</v>
       </c>
       <c r="L30" t="n">
         <v>52.59</v>
@@ -31525,7 +31387,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K32" t="n">
-        <v>2.43</v>
+        <v>2.84</v>
       </c>
       <c r="L32" t="n">
         <v>68.95999999999999</v>
@@ -31585,7 +31447,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K33" t="n">
-        <v>1.08</v>
+        <v>1.51</v>
       </c>
       <c r="L33" t="n">
         <v>36.81</v>
@@ -31645,7 +31507,7 @@
         <v>0.03</v>
       </c>
       <c r="K34" t="n">
-        <v>2.44</v>
+        <v>0.91</v>
       </c>
       <c r="L34" t="n">
         <v>43.87</v>
@@ -31705,7 +31567,7 @@
         <v>0.09</v>
       </c>
       <c r="K35" t="n">
-        <v>5.94</v>
+        <v>2.81</v>
       </c>
       <c r="L35" t="n">
         <v>57.85</v>
@@ -31765,7 +31627,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="K36" t="n">
-        <v>2.03</v>
+        <v>2.37</v>
       </c>
       <c r="L36" t="n">
         <v>57.97</v>
@@ -31825,7 +31687,7 @@
         <v>0.09</v>
       </c>
       <c r="K37" t="n">
-        <v>16.05</v>
+        <v>7.22</v>
       </c>
       <c r="L37" t="n">
         <v>148.48</v>
@@ -31981,7 +31843,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.92</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>79.3</v>
@@ -32041,7 +31903,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>2.39</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>78.73</v>
@@ -32101,7 +31963,7 @@
         <v>0.01</v>
       </c>
       <c r="K4" t="n">
-        <v>1.17</v>
+        <v>0.39</v>
       </c>
       <c r="L4" t="n">
         <v>67.51000000000001</v>
@@ -32161,7 +32023,7 @@
         <v>0.01</v>
       </c>
       <c r="K5" t="n">
-        <v>0.61</v>
+        <v>0.2</v>
       </c>
       <c r="L5" t="n">
         <v>35.4</v>
@@ -32221,7 +32083,7 @@
         <v>0.01</v>
       </c>
       <c r="K6" t="n">
-        <v>1.4</v>
+        <v>0.47</v>
       </c>
       <c r="L6" t="n">
         <v>80.76000000000001</v>

</xml_diff>